<commit_message>
Anchor seeded dates to the generation day so none fall in the future
</commit_message>
<xml_diff>
--- a/Chowly - Seed Data.xlsx
+++ b/Chowly - Seed Data.xlsx
@@ -908,12 +908,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-01 17:08</t>
+          <t>2026-08-29 17:08</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-01 17:52</t>
+          <t>2026-08-29 17:52</t>
         </is>
       </c>
     </row>
@@ -940,12 +940,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-01 12:06</t>
+          <t>2026-08-29 12:06</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-01 13:01</t>
+          <t>2026-08-29 13:01</t>
         </is>
       </c>
     </row>
@@ -972,12 +972,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-01 16:32</t>
+          <t>2026-08-29 16:32</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-01 17:23</t>
+          <t>2026-08-29 17:23</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-01 14:10</t>
+          <t>2026-08-29 14:10</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-01 14:59</t>
+          <t>2026-08-29 14:59</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-01 17:29</t>
+          <t>2026-08-29 17:29</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-01 17:58</t>
+          <t>2026-08-29 17:58</t>
         </is>
       </c>
     </row>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-02 20:19</t>
+          <t>2026-08-30 20:19</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-02 21:03</t>
+          <t>2026-08-30 21:03</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-02 14:53</t>
+          <t>2026-08-30 14:53</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-02 15:45</t>
+          <t>2026-08-30 15:45</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-02 15:04</t>
+          <t>2026-08-30 15:04</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-02 15:52</t>
+          <t>2026-08-30 15:52</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-02 16:08</t>
+          <t>2026-08-30 16:08</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-02 16:45</t>
+          <t>2026-08-30 16:45</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1196,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-02 19:53</t>
+          <t>2026-08-30 19:53</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-02 20:18</t>
+          <t>2026-08-30 20:18</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1228,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-03 16:41</t>
+          <t>2026-08-31 16:41</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-08-31 17:37</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-03 20:45</t>
+          <t>2026-08-31 20:45</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-03 21:03</t>
+          <t>2026-08-31 21:03</t>
         </is>
       </c>
     </row>
@@ -1284,12 +1284,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-03 20:38</t>
+          <t>2026-08-31 20:38</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-03 20:59</t>
+          <t>2026-08-31 20:59</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1312,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-03 13:25</t>
+          <t>2026-08-31 13:25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-03 14:16</t>
+          <t>2026-08-31 14:16</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-03 17:36</t>
+          <t>2026-08-31 17:36</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-04 18:24</t>
+          <t>2026-09-01 18:24</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1400,12 +1400,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-04 19:15</t>
+          <t>2026-09-01 19:15</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-04 19:42</t>
+          <t>2026-09-01 19:42</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-04 13:26</t>
+          <t>2026-09-01 13:26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-04 14:21</t>
+          <t>2026-09-01 14:21</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-04 15:44</t>
+          <t>2026-09-01 15:44</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-04 17:00</t>
+          <t>2026-09-01 17:00</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-04 17:11</t>
+          <t>2026-09-01 17:11</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-04 18:11</t>
+          <t>2026-09-01 18:11</t>
         </is>
       </c>
     </row>
@@ -1524,12 +1524,12 @@
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-04 20:57</t>
+          <t>2026-09-01 20:57</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-04 21:51</t>
+          <t>2026-09-01 21:51</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-05 12:27</t>
+          <t>2026-09-02 12:27</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-05 12:35</t>
+          <t>2026-09-02 12:35</t>
         </is>
       </c>
     </row>
@@ -1588,12 +1588,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-05 14:39</t>
+          <t>2026-09-02 14:39</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-05 15:33</t>
+          <t>2026-09-02 15:33</t>
         </is>
       </c>
     </row>
@@ -1620,12 +1620,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-05 17:08</t>
+          <t>2026-09-02 17:08</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-05 17:36</t>
+          <t>2026-09-02 17:36</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-05 16:52</t>
+          <t>2026-09-02 16:52</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-05 15:06</t>
+          <t>2026-09-02 15:06</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1704,12 +1704,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-05 12:10</t>
+          <t>2026-09-02 12:10</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-05 13:01</t>
+          <t>2026-09-02 13:01</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-06 13:28</t>
+          <t>2026-09-03 13:28</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-06 14:01</t>
+          <t>2026-09-03 14:01</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-06 20:39</t>
+          <t>2026-09-03 20:39</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-06 21:37</t>
+          <t>2026-09-03 21:37</t>
         </is>
       </c>
     </row>
@@ -1800,12 +1800,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-06 17:15</t>
+          <t>2026-09-03 17:15</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-06 17:51</t>
+          <t>2026-09-03 17:51</t>
         </is>
       </c>
     </row>
@@ -1832,12 +1832,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-06 12:21</t>
+          <t>2026-09-03 12:21</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-06 13:31</t>
+          <t>2026-09-03 13:31</t>
         </is>
       </c>
     </row>
@@ -1864,12 +1864,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-06 12:29</t>
+          <t>2026-09-03 12:29</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-06 13:08</t>
+          <t>2026-09-03 13:08</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-07 14:38</t>
+          <t>2026-09-04 14:38</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-07 15:37</t>
+          <t>2026-09-04 15:37</t>
         </is>
       </c>
     </row>
@@ -1924,12 +1924,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-07 17:10</t>
+          <t>2026-09-04 17:10</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-07 17:48</t>
+          <t>2026-09-04 17:48</t>
         </is>
       </c>
     </row>
@@ -1952,12 +1952,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-07 12:32</t>
+          <t>2026-09-04 12:32</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-07 12:40</t>
+          <t>2026-09-04 12:40</t>
         </is>
       </c>
     </row>
@@ -1984,12 +1984,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-07 18:50</t>
+          <t>2026-09-04 18:50</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-07 19:17</t>
+          <t>2026-09-04 19:17</t>
         </is>
       </c>
     </row>
@@ -2016,12 +2016,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-07 19:28</t>
+          <t>2026-09-04 19:28</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-07 20:04</t>
+          <t>2026-09-04 20:04</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-07 16:22</t>
+          <t>2026-09-04 16:22</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2072,12 +2072,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-08 18:18</t>
+          <t>2026-09-05 18:18</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-08 19:22</t>
+          <t>2026-09-05 19:22</t>
         </is>
       </c>
     </row>
@@ -2104,12 +2104,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-08 15:29</t>
+          <t>2026-09-05 15:29</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-08 16:00</t>
+          <t>2026-09-05 16:00</t>
         </is>
       </c>
     </row>
@@ -2136,12 +2136,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-08 16:17</t>
+          <t>2026-09-05 16:17</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-08 16:36</t>
+          <t>2026-09-05 16:36</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-01 17:57</t>
+          <t>2026-08-29 17:57</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-01 13:04</t>
+          <t>2026-08-29 13:04</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2307,7 +2307,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-01 17:24</t>
+          <t>2026-08-29 17:24</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-01 15:05</t>
+          <t>2026-08-29 15:05</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-01 18:01</t>
+          <t>2026-08-29 18:01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-02 15:49</t>
+          <t>2026-08-30 15:49</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-02 15:58</t>
+          <t>2026-08-30 15:58</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-02 16:48</t>
+          <t>2026-08-30 16:48</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-03 14:19</t>
+          <t>2026-08-31 14:19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-04 19:43</t>
+          <t>2026-09-01 19:43</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-04 14:23</t>
+          <t>2026-09-01 14:23</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2595,7 +2595,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-04 17:06</t>
+          <t>2026-09-01 17:06</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-04 18:15</t>
+          <t>2026-09-01 18:15</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-04 21:56</t>
+          <t>2026-09-01 21:56</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-05 15:38</t>
+          <t>2026-09-02 15:38</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-05 17:39</t>
+          <t>2026-09-02 17:39</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03</t>
+          <t>2026-09-02 13:03</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-06 14:06</t>
+          <t>2026-09-03 14:06</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-06 21:43</t>
+          <t>2026-09-03 21:43</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-06 13:32</t>
+          <t>2026-09-03 13:32</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-07 15:39</t>
+          <t>2026-09-04 15:39</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-07 17:49</t>
+          <t>2026-09-04 17:49</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2947,7 +2947,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-07 20:05</t>
+          <t>2026-09-04 20:05</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-08 19:28</t>
+          <t>2026-09-05 19:28</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-08 16:06</t>
+          <t>2026-09-05 16:06</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-01 18:02</t>
+          <t>2026-08-29 18:02</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-01 13:09</t>
+          <t>2026-08-29 13:09</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3181,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-01 17:32</t>
+          <t>2026-08-29 17:32</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-01 15:07</t>
+          <t>2026-08-29 15:07</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-01 18:03</t>
+          <t>2026-08-29 18:03</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3271,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-02 21:06</t>
+          <t>2026-08-30 21:06</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-02 15:52</t>
+          <t>2026-08-30 15:52</t>
         </is>
       </c>
     </row>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-02 15:54</t>
+          <t>2026-08-30 15:54</t>
         </is>
       </c>
     </row>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-02 16:54</t>
+          <t>2026-08-30 16:54</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-09-02 20:21</t>
+          <t>2026-08-30 20:21</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-03 17:44</t>
+          <t>2026-08-31 17:44</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-03 21:10</t>
+          <t>2026-08-31 21:10</t>
         </is>
       </c>
     </row>
@@ -3481,7 +3481,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-03 21:03</t>
+          <t>2026-08-31 21:03</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-09-03 14:26</t>
+          <t>2026-08-31 14:26</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-03 18:24</t>
+          <t>2026-08-31 18:24</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-04 18:50</t>
+          <t>2026-09-01 18:50</t>
         </is>
       </c>
     </row>
@@ -3601,7 +3601,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-04 19:48</t>
+          <t>2026-09-01 19:48</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-04 14:23</t>
+          <t>2026-09-01 14:23</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-04 17:05</t>
+          <t>2026-09-01 17:05</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-04 18:21</t>
+          <t>2026-09-01 18:21</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-04 21:59</t>
+          <t>2026-09-01 21:59</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-05 12:41</t>
+          <t>2026-09-02 12:41</t>
         </is>
       </c>
     </row>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-05 15:37</t>
+          <t>2026-09-02 15:37</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3811,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-05 17:39</t>
+          <t>2026-09-02 17:39</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-05 17:41</t>
+          <t>2026-09-02 17:41</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-05 15:46</t>
+          <t>2026-09-02 15:46</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-05 13:07</t>
+          <t>2026-09-02 13:07</t>
         </is>
       </c>
     </row>
@@ -3931,7 +3931,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-06 14:03</t>
+          <t>2026-09-03 14:03</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3961,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-06 21:45</t>
+          <t>2026-09-03 21:45</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-06 17:58</t>
+          <t>2026-09-03 17:58</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-06 13:39</t>
+          <t>2026-09-03 13:39</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-07 15:41</t>
+          <t>2026-09-04 15:41</t>
         </is>
       </c>
     </row>
@@ -4081,7 +4081,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-07 17:54</t>
+          <t>2026-09-04 17:54</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-07 20:12</t>
+          <t>2026-09-04 20:12</t>
         </is>
       </c>
     </row>
@@ -4141,7 +4141,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-08 19:28</t>
+          <t>2026-09-05 19:28</t>
         </is>
       </c>
     </row>
@@ -4171,7 +4171,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-08 16:03</t>
+          <t>2026-09-05 16:03</t>
         </is>
       </c>
     </row>
@@ -4282,12 +4282,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CHW-20260901-0001</t>
+          <t>CHW-20260829-0001</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-09-01 17:57</t>
+          <t>2026-08-29 17:57</t>
         </is>
       </c>
     </row>
@@ -4317,12 +4317,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CHW-20260901-0002</t>
+          <t>CHW-20260829-0002</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-09-01 13:11</t>
+          <t>2026-08-29 13:11</t>
         </is>
       </c>
     </row>
@@ -4352,12 +4352,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CHW-20260901-0003</t>
+          <t>CHW-20260829-0003</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-09-01 17:39</t>
+          <t>2026-08-29 17:39</t>
         </is>
       </c>
     </row>
@@ -4387,12 +4387,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CHW-20260901-0004</t>
+          <t>CHW-20260829-0004</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-09-01 15:18</t>
+          <t>2026-08-29 15:18</t>
         </is>
       </c>
     </row>
@@ -4422,12 +4422,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CHW-20260901-0005</t>
+          <t>CHW-20260829-0005</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-09-01 18:16</t>
+          <t>2026-08-29 18:16</t>
         </is>
       </c>
     </row>
@@ -4457,12 +4457,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>CHW-20260901-0006</t>
+          <t>CHW-20260829-0006</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-09-02 15:59</t>
+          <t>2026-08-30 15:59</t>
         </is>
       </c>
     </row>
@@ -4492,12 +4492,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CHW-20260901-0007</t>
+          <t>CHW-20260829-0007</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-09-02 16:10</t>
+          <t>2026-08-30 16:10</t>
         </is>
       </c>
     </row>
@@ -4527,12 +4527,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>CHW-20260901-0008</t>
+          <t>CHW-20260829-0008</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-09-02 17:01</t>
+          <t>2026-08-30 17:01</t>
         </is>
       </c>
     </row>
@@ -4562,12 +4562,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>CHW-20260901-0009</t>
+          <t>CHW-20260829-0009</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-09-02 20:34</t>
+          <t>2026-08-30 20:34</t>
         </is>
       </c>
     </row>
@@ -4597,12 +4597,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>CHW-20260901-0010</t>
+          <t>CHW-20260829-0010</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-03 17:42</t>
+          <t>2026-08-31 17:42</t>
         </is>
       </c>
     </row>
@@ -4632,12 +4632,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>CHW-20260901-0011</t>
+          <t>CHW-20260829-0011</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-03 21:14</t>
+          <t>2026-08-31 21:14</t>
         </is>
       </c>
     </row>
@@ -4667,12 +4667,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>CHW-20260901-0012</t>
+          <t>CHW-20260829-0012</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-09-03 14:35</t>
+          <t>2026-08-31 14:35</t>
         </is>
       </c>
     </row>
@@ -4702,12 +4702,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>CHW-20260901-0013</t>
+          <t>CHW-20260829-0013</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-04 19:49</t>
+          <t>2026-09-01 19:49</t>
         </is>
       </c>
     </row>
@@ -4737,12 +4737,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CHW-20260901-0014</t>
+          <t>CHW-20260829-0014</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-04 17:14</t>
+          <t>2026-09-01 17:14</t>
         </is>
       </c>
     </row>
@@ -4772,12 +4772,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CHW-20260901-0015</t>
+          <t>CHW-20260829-0015</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-04 18:21</t>
+          <t>2026-09-01 18:21</t>
         </is>
       </c>
     </row>
@@ -4807,12 +4807,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CHW-20260901-0016</t>
+          <t>CHW-20260829-0016</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-04 21:56</t>
+          <t>2026-09-01 21:56</t>
         </is>
       </c>
     </row>
@@ -4842,12 +4842,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CHW-20260901-0017</t>
+          <t>CHW-20260829-0017</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-05 12:41</t>
+          <t>2026-09-02 12:41</t>
         </is>
       </c>
     </row>
@@ -4877,12 +4877,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CHW-20260901-0018</t>
+          <t>CHW-20260829-0018</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-09-05 15:42</t>
+          <t>2026-09-02 15:42</t>
         </is>
       </c>
     </row>
@@ -4912,12 +4912,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CHW-20260901-0019</t>
+          <t>CHW-20260829-0019</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-09-05 17:42</t>
+          <t>2026-09-02 17:42</t>
         </is>
       </c>
     </row>
@@ -4947,12 +4947,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CHW-20260901-0020</t>
+          <t>CHW-20260829-0020</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-09-06 14:10</t>
+          <t>2026-09-03 14:10</t>
         </is>
       </c>
     </row>
@@ -4982,12 +4982,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CHW-20260901-0021</t>
+          <t>CHW-20260829-0021</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-09-06 21:44</t>
+          <t>2026-09-03 21:44</t>
         </is>
       </c>
     </row>
@@ -5017,12 +5017,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CHW-20260901-0022</t>
+          <t>CHW-20260829-0022</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-09-06 13:41</t>
+          <t>2026-09-03 13:41</t>
         </is>
       </c>
     </row>
@@ -5052,12 +5052,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CHW-20260901-0023</t>
+          <t>CHW-20260829-0023</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-09-06 13:25</t>
+          <t>2026-09-03 13:25</t>
         </is>
       </c>
     </row>
@@ -5087,12 +5087,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CHW-20260901-0024</t>
+          <t>CHW-20260829-0024</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-09-07 17:56</t>
+          <t>2026-09-04 17:56</t>
         </is>
       </c>
     </row>
@@ -5122,12 +5122,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CHW-20260901-0025</t>
+          <t>CHW-20260829-0025</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-09-07 12:47</t>
+          <t>2026-09-04 12:47</t>
         </is>
       </c>
     </row>
@@ -5157,12 +5157,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CHW-20260901-0026</t>
+          <t>CHW-20260829-0026</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-09-07 19:26</t>
+          <t>2026-09-04 19:26</t>
         </is>
       </c>
     </row>
@@ -5192,12 +5192,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CHW-20260901-0027</t>
+          <t>CHW-20260829-0027</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-09-07 20:15</t>
+          <t>2026-09-04 20:15</t>
         </is>
       </c>
     </row>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CHW-20260901-0028</t>
+          <t>CHW-20260829-0028</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-09-08 19:25</t>
+          <t>2026-09-05 19:25</t>
         </is>
       </c>
     </row>
@@ -5262,12 +5262,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CHW-20260901-0029</t>
+          <t>CHW-20260829-0029</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-09-08 16:04</t>
+          <t>2026-09-05 16:04</t>
         </is>
       </c>
     </row>
@@ -5297,12 +5297,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>CHW-20260901-0030</t>
+          <t>CHW-20260829-0030</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-09-08 16:45</t>
+          <t>2026-09-05 16:45</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2025-11-16</t>
         </is>
       </c>
     </row>
@@ -7052,7 +7052,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2025-11-11</t>
         </is>
       </c>
     </row>
@@ -7348,7 +7348,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-12-01</t>
+          <t>2025-12-01</t>
         </is>
       </c>
     </row>
@@ -7496,7 +7496,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2025-10-18</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2025-09-17</t>
         </is>
       </c>
     </row>
@@ -7681,7 +7681,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2025-09-03</t>
         </is>
       </c>
     </row>
@@ -8088,7 +8088,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2025-08-26</t>
         </is>
       </c>
     </row>
@@ -8347,7 +8347,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2025-10-10</t>
         </is>
       </c>
     </row>
@@ -8421,7 +8421,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-12-17</t>
+          <t>2025-12-17</t>
         </is>
       </c>
     </row>
@@ -19682,7 +19682,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-01 17:05</t>
+          <t>2026-08-29 17:05</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -19723,7 +19723,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-01 12:15</t>
+          <t>2026-08-29 12:15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -19764,7 +19764,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-01 12:03</t>
+          <t>2026-08-29 12:03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -19805,7 +19805,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-01 16:31</t>
+          <t>2026-08-29 16:31</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-09-01 14:06</t>
+          <t>2026-08-29 14:06</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -19887,7 +19887,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-01 17:27</t>
+          <t>2026-08-29 17:27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -19928,7 +19928,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-02 20:16</t>
+          <t>2026-08-30 20:16</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -19969,7 +19969,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-02 14:50</t>
+          <t>2026-08-30 14:50</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -20010,7 +20010,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-02 15:01</t>
+          <t>2026-08-30 15:01</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -20051,7 +20051,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-02 13:30</t>
+          <t>2026-08-30 13:30</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-02 16:05</t>
+          <t>2026-08-30 16:05</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -20133,7 +20133,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-02 19:49</t>
+          <t>2026-08-30 19:49</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -20174,7 +20174,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-03 16:38</t>
+          <t>2026-08-31 16:38</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-03 20:43</t>
+          <t>2026-08-31 20:43</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -20256,7 +20256,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-03 20:37</t>
+          <t>2026-08-31 20:37</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -20297,7 +20297,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-03 18:42</t>
+          <t>2026-08-31 18:42</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -20338,7 +20338,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-03 13:23</t>
+          <t>2026-08-31 13:23</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -20379,7 +20379,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-03 17:34</t>
+          <t>2026-08-31 17:34</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -20420,7 +20420,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-04 18:23</t>
+          <t>2026-09-01 18:23</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -20461,7 +20461,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-04 19:11</t>
+          <t>2026-09-01 19:11</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -20502,7 +20502,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-04 13:24</t>
+          <t>2026-09-01 13:24</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -20543,7 +20543,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-04 15:42</t>
+          <t>2026-09-01 15:42</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -20584,7 +20584,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-04 17:10</t>
+          <t>2026-09-01 17:10</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -20625,7 +20625,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-04 20:56</t>
+          <t>2026-09-01 20:56</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -20666,7 +20666,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-05 12:23</t>
+          <t>2026-09-02 12:23</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -20707,7 +20707,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-05 14:37</t>
+          <t>2026-09-02 14:37</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -20748,7 +20748,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-05 17:07</t>
+          <t>2026-09-02 17:07</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -20789,7 +20789,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-05 16:48</t>
+          <t>2026-09-02 16:48</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -20830,7 +20830,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-05 15:02</t>
+          <t>2026-09-02 15:02</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -20871,7 +20871,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-05 12:08</t>
+          <t>2026-09-02 12:08</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -20912,7 +20912,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-06 13:24</t>
+          <t>2026-09-03 13:24</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -20953,7 +20953,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-06 18:46</t>
+          <t>2026-09-03 18:46</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -20994,7 +20994,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-06 20:38</t>
+          <t>2026-09-03 20:38</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -21035,7 +21035,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-06 17:14</t>
+          <t>2026-09-03 17:14</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -21076,7 +21076,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-06 12:17</t>
+          <t>2026-09-03 12:17</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -21117,7 +21117,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-06 12:26</t>
+          <t>2026-09-03 12:26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -21158,7 +21158,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-07 14:36</t>
+          <t>2026-09-04 14:36</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -21199,7 +21199,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-07 17:06</t>
+          <t>2026-09-04 17:06</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -21240,7 +21240,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-07 12:30</t>
+          <t>2026-09-04 12:30</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -21281,7 +21281,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-07 18:47</t>
+          <t>2026-09-04 18:47</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -21322,7 +21322,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-07 19:27</t>
+          <t>2026-09-04 19:27</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21363,7 +21363,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-07 16:21</t>
+          <t>2026-09-04 16:21</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21404,7 +21404,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-08 18:14</t>
+          <t>2026-09-05 18:14</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -21445,7 +21445,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-09-08 15:25</t>
+          <t>2026-09-05 15:25</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -21486,7 +21486,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-09-08 16:14</t>
+          <t>2026-09-05 16:14</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">

</xml_diff>

<commit_message>
Keep in-flight orders current and stop ratings on unserved orders
</commit_message>
<xml_diff>
--- a/Chowly - Seed Data.xlsx
+++ b/Chowly - Seed Data.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="19">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-31 17:36</t>
+          <t>2026-09-06 23:24</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-01 18:24</t>
+          <t>2026-09-06 23:26</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1400,12 +1400,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-01 19:15</t>
+          <t>2026-09-01 16:05</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-01 19:42</t>
+          <t>2026-09-01 16:16</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-01 13:26</t>
+          <t>2026-09-01 18:19</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-01 14:21</t>
+          <t>2026-09-01 19:00</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-01 15:44</t>
+          <t>2026-09-01 17:24</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-01 17:00</t>
+          <t>2026-09-01 18:12</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-01 17:11</t>
+          <t>2026-09-01 20:34</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-01 18:11</t>
+          <t>2026-09-01 21:21</t>
         </is>
       </c>
     </row>
@@ -1521,15 +1521,19 @@
           <t>S247</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>S248</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-01 20:57</t>
+          <t>2026-09-01 19:08</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-01 21:51</t>
+          <t>2026-09-01 20:13</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1560,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-02 12:27</t>
+          <t>2026-09-02 15:39</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-02 12:35</t>
+          <t>2026-09-02 15:53</t>
         </is>
       </c>
     </row>
@@ -1588,12 +1592,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-02 14:39</t>
+          <t>2026-09-02 16:33</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-02 15:33</t>
+          <t>2026-09-02 17:42</t>
         </is>
       </c>
     </row>
@@ -1613,19 +1617,15 @@
           <t>S211</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>S212</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-02 17:08</t>
+          <t>2026-09-02 16:59</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-02 17:36</t>
+          <t>2026-09-02 17:29</t>
         </is>
       </c>
     </row>
@@ -1645,14 +1645,10 @@
           <t>S215</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>S216</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-02 16:52</t>
+          <t>2026-09-06 23:15</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1680,7 +1676,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-02 15:06</t>
+          <t>2026-09-06 23:45</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1696,7 +1692,11 @@
           <t>ORD030</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>S223</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>S224</t>
@@ -1704,12 +1704,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-02 12:10</t>
+          <t>2026-09-02 15:06</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-02 13:01</t>
+          <t>2026-09-02 16:22</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-03 13:28</t>
+          <t>2026-09-03 14:03</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-03 14:01</t>
+          <t>2026-09-03 14:24</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-03 20:39</t>
+          <t>2026-09-03 20:15</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-03 21:37</t>
+          <t>2026-09-03 20:40</t>
         </is>
       </c>
     </row>
@@ -1788,11 +1788,7 @@
           <t>ORD034</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>S239</t>
-        </is>
-      </c>
+      <c r="C35" t="inlineStr"/>
       <c r="D35" t="inlineStr">
         <is>
           <t>S240</t>
@@ -1800,12 +1796,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-03 17:15</t>
+          <t>2026-09-03 16:55</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-03 17:51</t>
+          <t>2026-09-03 17:13</t>
         </is>
       </c>
     </row>
@@ -1825,19 +1821,15 @@
           <t>S243</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>S244</t>
-        </is>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-03 12:21</t>
+          <t>2026-09-03 19:09</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-03 13:31</t>
+          <t>2026-09-03 20:13</t>
         </is>
       </c>
     </row>
@@ -1857,19 +1849,15 @@
           <t>S247</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>S248</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-03 12:29</t>
+          <t>2026-09-03 15:05</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-03 13:08</t>
+          <t>2026-09-03 15:50</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1884,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-04 14:38</t>
+          <t>2026-09-04 17:29</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-04 15:37</t>
+          <t>2026-09-04 18:21</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1904,11 @@
           <t>ORD038</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>S202</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>S203</t>
@@ -1924,12 +1916,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-04 17:10</t>
+          <t>2026-09-04 13:50</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-04 17:48</t>
+          <t>2026-09-04 14:49</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1936,11 @@
           <t>ORD039</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>S211</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>S212</t>
@@ -1952,12 +1948,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-04 12:32</t>
+          <t>2026-09-04 20:49</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-04 12:40</t>
+          <t>2026-09-04 21:05</t>
         </is>
       </c>
     </row>
@@ -1972,11 +1968,7 @@
           <t>ORD040</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>S215</t>
-        </is>
-      </c>
+      <c r="C41" t="inlineStr"/>
       <c r="D41" t="inlineStr">
         <is>
           <t>S216</t>
@@ -1984,12 +1976,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-04 18:50</t>
+          <t>2026-09-04 16:11</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-04 19:17</t>
+          <t>2026-09-04 16:25</t>
         </is>
       </c>
     </row>
@@ -2004,11 +1996,7 @@
           <t>ORD041</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>S219</t>
-        </is>
-      </c>
+      <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr">
         <is>
           <t>S220</t>
@@ -2016,12 +2004,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-04 19:28</t>
+          <t>2026-09-04 19:54</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-04 20:04</t>
+          <t>2026-09-04 20:39</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2032,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-04 16:22</t>
+          <t>2026-09-06 23:37</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2072,12 +2060,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-05 18:18</t>
+          <t>2026-09-05 13:38</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-05 19:22</t>
+          <t>2026-09-05 14:45</t>
         </is>
       </c>
     </row>
@@ -2097,19 +2085,15 @@
           <t>S231</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>S232</t>
-        </is>
-      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-05 15:29</t>
+          <t>2026-09-05 19:22</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-05 16:00</t>
+          <t>2026-09-05 20:24</t>
         </is>
       </c>
     </row>
@@ -2129,19 +2113,15 @@
           <t>S235</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>S236</t>
-        </is>
-      </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-05 16:17</t>
+          <t>2026-09-05 17:46</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-05 16:36</t>
+          <t>2026-09-05 18:16</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2184,7 +2164,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>25 records</t>
+          <t>22 records</t>
         </is>
       </c>
     </row>
@@ -2516,27 +2496,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ORD020</t>
+          <t>ORD021</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C017</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Order took far longer than the quoted time</t>
+          <t>We waited well past the estimated wait</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-01 19:43</t>
+          <t>2026-09-01 19:05</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2548,22 +2528,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ORD021</t>
+          <t>ORD022</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>C014</t>
+          <t>C013</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Order took far longer than the quoted time</t>
+          <t>Drinks came very late</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-01 14:23</t>
+          <t>2026-09-01 18:17</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2580,12 +2560,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ORD022</t>
+          <t>ORD023</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C022</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2595,7 +2575,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-01 17:06</t>
+          <t>2026-09-01 21:23</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2612,27 +2592,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ORD023</t>
+          <t>ORD024</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C005</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Serious delay before the food arrived</t>
+          <t>We waited well past the estimated wait</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-01 18:15</t>
+          <t>2026-09-01 20:18</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2644,22 +2624,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ORD024</t>
+          <t>ORD026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C021</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Serious delay before the food arrived</t>
+          <t>We waited well past the estimated wait</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-01 21:56</t>
+          <t>2026-09-02 17:46</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2676,22 +2656,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ORD026</t>
+          <t>ORD030</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>C022</t>
+          <t>C019</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Serious delay before the food arrived</t>
+          <t>Order took far longer than the quoted time</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-02 15:38</t>
+          <t>2026-09-02 16:26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2708,7 +2688,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ORD028</t>
+          <t>ORD033</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2723,12 +2703,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-02 17:39</t>
+          <t>2026-09-03 20:44</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2740,12 +2720,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ORD030</t>
+          <t>ORD035</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C015</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2755,12 +2735,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-02 13:03</t>
+          <t>2026-09-03 20:18</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2772,27 +2752,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ORD031</t>
+          <t>ORD037</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>C021</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Serious delay before the food arrived</t>
+          <t>Order took far longer than the quoted time</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-03 14:06</t>
+          <t>2026-09-04 18:26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2784,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ORD033</t>
+          <t>ORD038</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2814,17 +2794,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>We waited well past the estimated wait</t>
+          <t>Order took far longer than the quoted time</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-03 21:43</t>
+          <t>2026-09-04 14:54</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Resolved</t>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2836,22 +2816,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ORD035</t>
+          <t>ORD041</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>C008</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Order took far longer than the quoted time</t>
+          <t>Drinks came very late</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-03 13:32</t>
+          <t>2026-09-04 20:42</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2868,12 +2848,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ORD037</t>
+          <t>ORD043</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2883,7 +2863,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-04 15:39</t>
+          <t>2026-09-05 14:46</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2900,7 +2880,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ORD038</t>
+          <t>ORD044</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2915,106 +2895,10 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-04 17:49</t>
+          <t>2026-09-05 20:26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
-        <is>
-          <t>Resolved</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>COM023</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>ORD041</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>C016</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Drinks came very late</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2026-09-04 20:05</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>COM024</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ORD043</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>C016</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Drinks came very late</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2026-09-05 19:28</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Resolved</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>COM025</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>ORD044</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>C017</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Order took far longer than the quoted time</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2026-09-05 16:06</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -3031,7 +2915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3059,7 +2943,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>36 records</t>
+          <t>33 records</t>
         </is>
       </c>
     </row>
@@ -3523,12 +3407,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ORD018</t>
+          <t>ORD020</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>C021</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -3536,12 +3420,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Will come again</t>
+          <t>Excellent service</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-08-31 18:24</t>
+          <t>2026-09-01 16:26</t>
         </is>
       </c>
     </row>
@@ -3553,25 +3437,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ORD019</t>
+          <t>ORD021</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C006</t>
+          <t>C017</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Lovely food</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-01 18:50</t>
+          <t>2026-09-01 19:03</t>
         </is>
       </c>
     </row>
@@ -3583,16 +3467,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ORD020</t>
+          <t>ORD022</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C013</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3601,7 +3485,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-01 19:48</t>
+          <t>2026-09-01 18:14</t>
         </is>
       </c>
     </row>
@@ -3613,12 +3497,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ORD021</t>
+          <t>ORD023</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>C014</t>
+          <t>C022</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -3626,12 +3510,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-01 14:23</t>
+          <t>2026-09-01 21:30</t>
         </is>
       </c>
     </row>
@@ -3643,16 +3527,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ORD022</t>
+          <t>ORD024</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C005</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3661,7 +3545,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-01 17:05</t>
+          <t>2026-09-01 20:16</t>
         </is>
       </c>
     </row>
@@ -3673,25 +3557,25 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ORD023</t>
+          <t>ORD025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Will come again</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-01 18:21</t>
+          <t>2026-09-02 15:57</t>
         </is>
       </c>
     </row>
@@ -3703,12 +3587,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ORD024</t>
+          <t>ORD026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C021</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -3716,12 +3600,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-01 21:59</t>
+          <t>2026-09-02 17:49</t>
         </is>
       </c>
     </row>
@@ -3733,25 +3617,25 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ORD025</t>
+          <t>ORD027</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>C015</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Lovely food</t>
+          <t>Excellent service</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-02 12:41</t>
+          <t>2026-09-02 17:37</t>
         </is>
       </c>
     </row>
@@ -3763,12 +3647,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ORD026</t>
+          <t>ORD030</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>C022</t>
+          <t>C019</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -3776,12 +3660,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-02 15:37</t>
+          <t>2026-09-02 16:24</t>
         </is>
       </c>
     </row>
@@ -3793,16 +3677,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ORD027</t>
+          <t>ORD031</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>C015</t>
+          <t>C023</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -3811,7 +3695,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-02 17:39</t>
+          <t>2026-09-03 14:30</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3707,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ORD028</t>
+          <t>ORD033</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3836,12 +3720,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-02 17:41</t>
+          <t>2026-09-03 20:46</t>
         </is>
       </c>
     </row>
@@ -3853,12 +3737,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ORD029</t>
+          <t>ORD034</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>C019</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -3866,12 +3750,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Very good</t>
+          <t>Will come again</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-02 15:46</t>
+          <t>2026-09-03 17:20</t>
         </is>
       </c>
     </row>
@@ -3883,12 +3767,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ORD030</t>
+          <t>ORD035</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C015</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -3901,7 +3785,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-02 13:07</t>
+          <t>2026-09-03 20:16</t>
         </is>
       </c>
     </row>
@@ -3913,25 +3797,25 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ORD031</t>
+          <t>ORD036</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>C021</t>
+          <t>C019</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Excellent service</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-03 14:03</t>
+          <t>2026-09-03 15:52</t>
         </is>
       </c>
     </row>
@@ -3943,12 +3827,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ORD033</t>
+          <t>ORD037</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -3956,12 +3840,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-03 21:45</t>
+          <t>2026-09-04 18:23</t>
         </is>
       </c>
     </row>
@@ -3973,25 +3857,25 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ORD034</t>
+          <t>ORD038</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>C009</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Very good</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-03 17:58</t>
+          <t>2026-09-04 14:51</t>
         </is>
       </c>
     </row>
@@ -4003,25 +3887,25 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ORD035</t>
+          <t>ORD041</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>C008</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Not happy with the delay</t>
+          <t>Long waiting time</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-03 13:39</t>
+          <t>2026-09-04 20:47</t>
         </is>
       </c>
     </row>
@@ -4033,16 +3917,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ORD037</t>
+          <t>ORD043</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -4051,7 +3935,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-04 15:41</t>
+          <t>2026-09-05 14:51</t>
         </is>
       </c>
     </row>
@@ -4063,7 +3947,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ORD038</t>
+          <t>ORD044</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4081,97 +3965,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-04 17:54</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>RT034</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>ORD041</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>C016</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Not happy with the delay</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>2026-09-04 20:12</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>RT035</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>ORD043</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>C016</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>2</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Long waiting time</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>2026-09-05 19:28</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>RT036</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>ORD044</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>C017</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Not happy with the delay</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>2026-09-05 16:03</t>
+          <t>2026-09-05 20:33</t>
         </is>
       </c>
     </row>
@@ -4688,11 +4482,11 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>64000</v>
+        <v>7000</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -4707,7 +4501,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-01 19:49</t>
+          <t>2026-09-01 16:32</t>
         </is>
       </c>
     </row>
@@ -4723,11 +4517,11 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>35000</v>
+        <v>23000</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Card</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -4742,7 +4536,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-01 17:14</t>
+          <t>2026-09-01 18:22</t>
         </is>
       </c>
     </row>
@@ -4758,11 +4552,11 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>25000</v>
+        <v>26500</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -4777,7 +4571,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-01 18:21</t>
+          <t>2026-09-01 21:29</t>
         </is>
       </c>
     </row>
@@ -4793,11 +4587,11 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>16000</v>
+        <v>57000</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Card</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -4812,7 +4606,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-01 21:56</t>
+          <t>2026-09-01 20:16</t>
         </is>
       </c>
     </row>
@@ -4828,11 +4622,11 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>8500</v>
+        <v>21000</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Card</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -4847,7 +4641,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-02 12:41</t>
+          <t>2026-09-02 16:01</t>
         </is>
       </c>
     </row>
@@ -4863,7 +4657,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9100</v>
+        <v>20500</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -4882,7 +4676,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-09-02 15:42</t>
+          <t>2026-09-02 17:51</t>
         </is>
       </c>
     </row>
@@ -4898,11 +4692,11 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>24500</v>
+        <v>27000</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -4917,7 +4711,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-09-02 17:42</t>
+          <t>2026-09-02 17:33</t>
         </is>
       </c>
     </row>
@@ -4933,11 +4727,11 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>37000</v>
+        <v>23500</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -4952,7 +4746,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-09-03 14:10</t>
+          <t>2026-09-03 14:27</t>
         </is>
       </c>
     </row>
@@ -4968,7 +4762,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>15800</v>
+        <v>10000</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -4987,7 +4781,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-09-03 21:44</t>
+          <t>2026-09-03 21:00</t>
         </is>
       </c>
     </row>
@@ -5003,7 +4797,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>10500</v>
+        <v>34500</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -5022,7 +4816,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-09-03 13:41</t>
+          <t>2026-09-03 20:30</t>
         </is>
       </c>
     </row>
@@ -5038,7 +4832,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>52500</v>
+        <v>41500</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -5057,7 +4851,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-09-03 13:25</t>
+          <t>2026-09-03 15:53</t>
         </is>
       </c>
     </row>
@@ -5073,7 +4867,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>19000</v>
+        <v>14500</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -5092,7 +4886,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-09-04 17:56</t>
+          <t>2026-09-04 15:09</t>
         </is>
       </c>
     </row>
@@ -5108,7 +4902,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>6800</v>
+        <v>20500</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -5127,7 +4921,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-09-04 12:47</t>
+          <t>2026-09-04 21:19</t>
         </is>
       </c>
     </row>
@@ -5143,11 +4937,11 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>15500</v>
+        <v>12000</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5162,7 +4956,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-09-04 19:26</t>
+          <t>2026-09-04 16:45</t>
         </is>
       </c>
     </row>
@@ -5178,7 +4972,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>28300</v>
+        <v>5600</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -5197,7 +4991,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-09-04 20:15</t>
+          <t>2026-09-04 20:43</t>
         </is>
       </c>
     </row>
@@ -5213,11 +5007,11 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>56000</v>
+        <v>24500</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5232,7 +5026,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-09-05 19:25</t>
+          <t>2026-09-05 14:52</t>
         </is>
       </c>
     </row>
@@ -5248,11 +5042,11 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>37000</v>
+        <v>48500</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Cash</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5267,7 +5061,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-09-05 16:04</t>
+          <t>2026-09-05 20:28</t>
         </is>
       </c>
     </row>
@@ -5283,11 +5077,11 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5302,7 +5096,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-09-05 16:45</t>
+          <t>2026-09-05 18:21</t>
         </is>
       </c>
     </row>
@@ -19723,7 +19517,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-29 12:15</t>
+          <t>2026-09-06 23:15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -20051,7 +19845,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-30 13:30</t>
+          <t>2026-09-06 23:32</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -20297,7 +20091,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-31 18:42</t>
+          <t>2026-09-06 23:43</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -20379,7 +20173,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-08-31 17:34</t>
+          <t>2026-09-06 23:22</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -20405,7 +20199,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>C006</t>
+          <t>C007</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -20415,12 +20209,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>S226</t>
+          <t>S229</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-01 18:23</t>
+          <t>2026-09-06 23:24</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -20432,7 +20226,7 @@
         <v>23</v>
       </c>
       <c r="H24" t="n">
-        <v>22000</v>
+        <v>30000</v>
       </c>
       <c r="I24" t="n">
         <v>4</v>
@@ -20446,7 +20240,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -20461,7 +20255,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-01 19:11</t>
+          <t>2026-09-01 16:01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -20470,10 +20264,10 @@
         </is>
       </c>
       <c r="G25" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H25" t="n">
-        <v>64000</v>
+        <v>7000</v>
       </c>
       <c r="I25" t="n">
         <v>1</v>
@@ -20487,7 +20281,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>C014</t>
+          <t>C017</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -20497,12 +20291,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>S234</t>
+          <t>S237</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-01 13:24</t>
+          <t>2026-09-01 18:16</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -20511,10 +20305,10 @@
         </is>
       </c>
       <c r="G26" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="H26" t="n">
-        <v>23900</v>
+        <v>22000</v>
       </c>
       <c r="I26" t="n">
         <v>5</v>
@@ -20528,7 +20322,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C013</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -20538,12 +20332,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>S238</t>
+          <t>S241</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-01 15:42</t>
+          <t>2026-09-01 17:20</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -20552,10 +20346,10 @@
         </is>
       </c>
       <c r="G27" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="H27" t="n">
-        <v>35000</v>
+        <v>23000</v>
       </c>
       <c r="I27" t="n">
         <v>17</v>
@@ -20569,7 +20363,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C022</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -20584,7 +20378,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-01 17:10</t>
+          <t>2026-09-01 20:30</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -20593,10 +20387,10 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H28" t="n">
-        <v>25000</v>
+        <v>26500</v>
       </c>
       <c r="I28" t="n">
         <v>5</v>
@@ -20610,7 +20404,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C005</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -20625,7 +20419,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-01 20:56</t>
+          <t>2026-09-01 19:05</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -20634,10 +20428,10 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H29" t="n">
-        <v>16000</v>
+        <v>57000</v>
       </c>
       <c r="I29" t="n">
         <v>6</v>
@@ -20651,7 +20445,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>C015</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -20661,12 +20455,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>S201</t>
+          <t>S204</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-02 12:23</t>
+          <t>2026-09-02 15:35</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -20675,10 +20469,10 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="H30" t="n">
-        <v>8500</v>
+        <v>21000</v>
       </c>
       <c r="I30" t="n">
         <v>11</v>
@@ -20692,7 +20486,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>C022</t>
+          <t>C021</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -20707,7 +20501,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-02 14:37</t>
+          <t>2026-09-02 16:30</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -20716,10 +20510,10 @@
         </is>
       </c>
       <c r="G31" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="H31" t="n">
-        <v>9100</v>
+        <v>20500</v>
       </c>
       <c r="I31" t="n">
         <v>4</v>
@@ -20733,7 +20527,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>C015</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -20748,7 +20542,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-02 17:07</t>
+          <t>2026-09-02 16:58</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -20757,10 +20551,10 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H32" t="n">
-        <v>24500</v>
+        <v>27000</v>
       </c>
       <c r="I32" t="n">
         <v>6</v>
@@ -20774,7 +20568,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C022</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -20789,7 +20583,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-02 16:48</t>
+          <t>2026-09-06 23:11</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -20798,10 +20592,10 @@
         </is>
       </c>
       <c r="G33" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="H33" t="n">
-        <v>19800</v>
+        <v>21000</v>
       </c>
       <c r="I33" t="n">
         <v>23</v>
@@ -20815,7 +20609,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>C019</t>
+          <t>C008</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -20825,12 +20619,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>S221</t>
+          <t>S218</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-02 15:02</t>
+          <t>2026-09-06 23:42</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -20839,10 +20633,10 @@
         </is>
       </c>
       <c r="G34" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H34" t="n">
-        <v>35000</v>
+        <v>30900</v>
       </c>
       <c r="I34" t="n">
         <v>8</v>
@@ -20856,7 +20650,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C019</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -20866,12 +20660,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>S222</t>
+          <t>S225</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-02 12:08</t>
+          <t>2026-09-02 15:02</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -20880,10 +20674,10 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="H35" t="n">
-        <v>66000</v>
+        <v>49500</v>
       </c>
       <c r="I35" t="n">
         <v>23</v>
@@ -20897,7 +20691,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>C021</t>
+          <t>C023</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -20912,7 +20706,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-03 13:24</t>
+          <t>2026-09-03 14:02</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -20921,10 +20715,10 @@
         </is>
       </c>
       <c r="G36" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H36" t="n">
-        <v>37000</v>
+        <v>23500</v>
       </c>
       <c r="I36" t="n">
         <v>19</v>
@@ -20938,7 +20732,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -20948,12 +20742,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>S233</t>
+          <t>S230</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-03 18:46</t>
+          <t>2026-09-06 23:33</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -20962,10 +20756,10 @@
         </is>
       </c>
       <c r="G37" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H37" t="n">
-        <v>21000</v>
+        <v>10000</v>
       </c>
       <c r="I37" t="n">
         <v>22</v>
@@ -20979,7 +20773,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -20989,12 +20783,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>S237</t>
+          <t>S234</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-03 20:38</t>
+          <t>2026-09-03 20:13</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -21003,10 +20797,10 @@
         </is>
       </c>
       <c r="G38" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="H38" t="n">
-        <v>15800</v>
+        <v>10000</v>
       </c>
       <c r="I38" t="n">
         <v>21</v>
@@ -21020,7 +20814,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>C009</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -21030,12 +20824,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>S241</t>
+          <t>S238</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-03 17:14</t>
+          <t>2026-09-03 16:54</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -21044,10 +20838,10 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H39" t="n">
-        <v>39500</v>
+        <v>18000</v>
       </c>
       <c r="I39" t="n">
         <v>8</v>
@@ -21061,7 +20855,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>C008</t>
+          <t>C015</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -21071,12 +20865,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>S242</t>
+          <t>S245</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-03 12:17</t>
+          <t>2026-09-03 19:08</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -21085,10 +20879,10 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="H40" t="n">
-        <v>10500</v>
+        <v>34500</v>
       </c>
       <c r="I40" t="n">
         <v>15</v>
@@ -21102,7 +20896,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C019</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -21117,7 +20911,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-03 12:26</t>
+          <t>2026-09-03 15:04</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -21129,7 +20923,7 @@
         <v>42</v>
       </c>
       <c r="H41" t="n">
-        <v>52500</v>
+        <v>41500</v>
       </c>
       <c r="I41" t="n">
         <v>2</v>
@@ -21143,7 +20937,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>C004</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -21153,12 +20947,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>S201</t>
+          <t>S208</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-04 14:36</t>
+          <t>2026-09-04 17:25</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -21167,10 +20961,10 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="H42" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="I42" t="n">
         <v>9</v>
@@ -21199,7 +20993,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-04 17:06</t>
+          <t>2026-09-04 13:49</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -21208,10 +21002,10 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H43" t="n">
-        <v>19000</v>
+        <v>14500</v>
       </c>
       <c r="I43" t="n">
         <v>11</v>
@@ -21225,7 +21019,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>C003</t>
+          <t>C012</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -21240,7 +21034,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-04 12:30</t>
+          <t>2026-09-04 20:48</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -21249,10 +21043,10 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="H44" t="n">
-        <v>6800</v>
+        <v>20500</v>
       </c>
       <c r="I44" t="n">
         <v>1</v>
@@ -21266,7 +21060,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>C009</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -21276,12 +21070,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>S214</t>
+          <t>S217</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-04 18:47</t>
+          <t>2026-09-04 16:09</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -21290,10 +21084,10 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="H45" t="n">
-        <v>15500</v>
+        <v>12000</v>
       </c>
       <c r="I45" t="n">
         <v>11</v>
@@ -21307,7 +21101,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>C016</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -21317,12 +21111,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>S221</t>
+          <t>S218</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-04 19:27</t>
+          <t>2026-09-04 19:52</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21331,10 +21125,10 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H46" t="n">
-        <v>28300</v>
+        <v>5600</v>
       </c>
       <c r="I46" t="n">
         <v>6</v>
@@ -21348,7 +21142,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -21358,12 +21152,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>S222</t>
+          <t>S225</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-04 16:21</t>
+          <t>2026-09-06 23:33</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21375,7 +21169,7 @@
         <v>16</v>
       </c>
       <c r="H47" t="n">
-        <v>43000</v>
+        <v>53000</v>
       </c>
       <c r="I47" t="n">
         <v>17</v>
@@ -21389,7 +21183,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>C016</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -21399,12 +21193,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>S226</t>
+          <t>S229</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-05 18:14</t>
+          <t>2026-09-05 13:35</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -21413,10 +21207,10 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H48" t="n">
-        <v>56000</v>
+        <v>24500</v>
       </c>
       <c r="I48" t="n">
         <v>11</v>
@@ -21430,7 +21224,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C017</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -21440,12 +21234,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>S230</t>
+          <t>S233</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-09-05 15:25</t>
+          <t>2026-09-05 19:18</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -21454,10 +21248,10 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="H49" t="n">
-        <v>37000</v>
+        <v>48500</v>
       </c>
       <c r="I49" t="n">
         <v>22</v>
@@ -21471,7 +21265,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>C016</t>
+          <t>C004</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -21481,12 +21275,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>S234</t>
+          <t>S237</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-09-05 16:14</t>
+          <t>2026-09-05 17:44</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21495,10 +21289,10 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H50" t="n">
-        <v>21000</v>
+        <v>22000</v>
       </c>
       <c r="I50" t="n">
         <v>12</v>
@@ -21515,7 +21309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E119"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21542,7 +21336,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>114 records</t>
+          <t>117 records</t>
         </is>
       </c>
     </row>
@@ -22568,17 +22362,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IT226</t>
+          <t>IT094</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>3500</v>
+        <v>7500</v>
       </c>
       <c r="E53" t="n">
-        <v>7000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="54">
@@ -22589,14 +22383,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IT094</t>
+          <t>IT221</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>7500</v>
+        <v>5000</v>
       </c>
       <c r="E54" t="n">
         <v>15000</v>
@@ -22610,17 +22404,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IT232</t>
+          <t>IT109</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>16000</v>
+        <v>4000</v>
       </c>
       <c r="E55" t="n">
-        <v>48000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="56">
@@ -22631,35 +22425,35 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IT109</t>
+          <t>IT236</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="E56" t="n">
-        <v>12000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ORD020</t>
+          <t>ORD021</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IT107</t>
+          <t>IT125</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="E57" t="n">
         <v>4000</v>
@@ -22673,59 +22467,59 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IT122</t>
+          <t>IT118</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D58" t="n">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="E58" t="n">
-        <v>3000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ORD021</t>
+          <t>ORD022</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>IT128</t>
+          <t>IT131</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>2300</v>
+        <v>9000</v>
       </c>
       <c r="E59" t="n">
-        <v>6900</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ORD021</t>
+          <t>ORD022</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IT124</t>
+          <t>IT138</t>
         </is>
       </c>
       <c r="C60" t="n">
         <v>2</v>
       </c>
       <c r="D60" t="n">
-        <v>7000</v>
+        <v>2000</v>
       </c>
       <c r="E60" t="n">
-        <v>14000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="61">
@@ -22736,59 +22530,59 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IT137</t>
+          <t>IT136</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D61" t="n">
-        <v>4000</v>
+        <v>5000</v>
       </c>
       <c r="E61" t="n">
-        <v>12000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ORD022</t>
+          <t>ORD023</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IT136</t>
+          <t>IT150</t>
         </is>
       </c>
       <c r="C62" t="n">
         <v>1</v>
       </c>
       <c r="D62" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="E62" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ORD022</t>
+          <t>ORD023</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>IT135</t>
+          <t>IT143</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D63" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="E63" t="n">
-        <v>18000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="64">
@@ -22799,38 +22593,38 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IT145</t>
+          <t>IT151</t>
         </is>
       </c>
       <c r="C64" t="n">
         <v>3</v>
       </c>
       <c r="D64" t="n">
-        <v>4000</v>
+        <v>6500</v>
       </c>
       <c r="E64" t="n">
-        <v>12000</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ORD023</t>
+          <t>ORD024</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>IT151</t>
+          <t>IT155</t>
         </is>
       </c>
       <c r="C65" t="n">
         <v>2</v>
       </c>
       <c r="D65" t="n">
-        <v>6500</v>
+        <v>8000</v>
       </c>
       <c r="E65" t="n">
-        <v>13000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="66">
@@ -22841,17 +22635,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>IT155</t>
+          <t>IT164</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D66" t="n">
-        <v>8000</v>
+        <v>17500</v>
       </c>
       <c r="E66" t="n">
-        <v>8000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="67">
@@ -22862,17 +22656,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>IT158</t>
+          <t>IT160</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D67" t="n">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="E67" t="n">
-        <v>8000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="68">
@@ -22883,17 +22677,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>IT034</t>
+          <t>IT030</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D68" t="n">
-        <v>3500</v>
+        <v>2500</v>
       </c>
       <c r="E68" t="n">
-        <v>3500</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="69">
@@ -22904,38 +22698,38 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>IT012</t>
+          <t>IT034</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="E69" t="n">
-        <v>5000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ORD026</t>
+          <t>ORD025</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>IT188</t>
+          <t>IT170</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>2500</v>
+        <v>3000</v>
       </c>
       <c r="E70" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="71">
@@ -22946,17 +22740,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>IT043</t>
+          <t>IT02</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D71" t="n">
-        <v>800</v>
+        <v>5000</v>
       </c>
       <c r="E71" t="n">
-        <v>2400</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="72">
@@ -22967,38 +22761,38 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IT180</t>
+          <t>IT024</t>
         </is>
       </c>
       <c r="C72" t="n">
         <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>1700</v>
+        <v>4500</v>
       </c>
       <c r="E72" t="n">
-        <v>1700</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ORD027</t>
+          <t>ORD026</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IT054</t>
+          <t>IT041</t>
         </is>
       </c>
       <c r="C73" t="n">
         <v>3</v>
       </c>
       <c r="D73" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="E73" t="n">
-        <v>7500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="74">
@@ -23009,17 +22803,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IT196</t>
+          <t>IT049</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>2</v>
       </c>
       <c r="D74" t="n">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="E74" t="n">
-        <v>6000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="75">
@@ -23030,38 +22824,38 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IT045</t>
+          <t>IT050</t>
         </is>
       </c>
       <c r="C75" t="n">
         <v>2</v>
       </c>
       <c r="D75" t="n">
-        <v>5500</v>
+        <v>3500</v>
       </c>
       <c r="E75" t="n">
-        <v>11000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ORD028</t>
+          <t>ORD027</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IT068</t>
+          <t>IT051</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D76" t="n">
-        <v>6500</v>
+        <v>5500</v>
       </c>
       <c r="E76" t="n">
-        <v>6500</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="77">
@@ -23072,17 +22866,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>IT203</t>
+          <t>IT058</t>
         </is>
       </c>
       <c r="C77" t="n">
         <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>1300</v>
+        <v>6500</v>
       </c>
       <c r="E77" t="n">
-        <v>1300</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="78">
@@ -23093,38 +22887,38 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IT062</t>
+          <t>IT059</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>6000</v>
+        <v>6500</v>
       </c>
       <c r="E78" t="n">
-        <v>12000</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ORD029</t>
+          <t>ORD028</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>IT208</t>
+          <t>IT060</t>
         </is>
       </c>
       <c r="C79" t="n">
         <v>2</v>
       </c>
       <c r="D79" t="n">
-        <v>2500</v>
+        <v>4000</v>
       </c>
       <c r="E79" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="80">
@@ -23135,416 +22929,416 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IT076</t>
+          <t>IT206</t>
         </is>
       </c>
       <c r="C80" t="n">
         <v>3</v>
       </c>
       <c r="D80" t="n">
-        <v>10000</v>
+        <v>3500</v>
       </c>
       <c r="E80" t="n">
-        <v>30000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ORD030</t>
+          <t>ORD029</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>IT215</t>
+          <t>IT071</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D81" t="n">
-        <v>6000</v>
+        <v>7500</v>
       </c>
       <c r="E81" t="n">
-        <v>6000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ORD030</t>
+          <t>ORD029</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IT218</t>
+          <t>IT077</t>
         </is>
       </c>
       <c r="C82" t="n">
         <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>20000</v>
+        <v>1800</v>
       </c>
       <c r="E82" t="n">
-        <v>60000</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ORD031</t>
+          <t>ORD030</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IT223</t>
+          <t>IT216</t>
         </is>
       </c>
       <c r="C83" t="n">
         <v>2</v>
       </c>
       <c r="D83" t="n">
-        <v>3500</v>
+        <v>6000</v>
       </c>
       <c r="E83" t="n">
-        <v>7000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ORD031</t>
+          <t>ORD030</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IT096</t>
+          <t>IT088</t>
         </is>
       </c>
       <c r="C84" t="n">
         <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>10000</v>
+        <v>12500</v>
       </c>
       <c r="E84" t="n">
-        <v>30000</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ORD032</t>
+          <t>ORD031</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>IT229</t>
+          <t>IT228</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D85" t="n">
-        <v>4000</v>
+        <v>2500</v>
       </c>
       <c r="E85" t="n">
-        <v>8000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ORD032</t>
+          <t>ORD031</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>IT108</t>
+          <t>IT226</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>1000</v>
+        <v>3500</v>
       </c>
       <c r="E86" t="n">
-        <v>1000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ORD032</t>
+          <t>ORD031</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IT234</t>
+          <t>IT095</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>4000</v>
+        <v>5500</v>
       </c>
       <c r="E87" t="n">
-        <v>12000</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ORD033</t>
+          <t>ORD032</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>IT127</t>
+          <t>IT108</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="E88" t="n">
-        <v>800</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ORD033</t>
+          <t>ORD032</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>IT121</t>
+          <t>IT230</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D89" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E89" t="n">
         <v>5000</v>
-      </c>
-      <c r="E89" t="n">
-        <v>15000</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ORD034</t>
+          <t>ORD032</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IT138</t>
+          <t>IT235</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D90" t="n">
         <v>2000</v>
       </c>
       <c r="E90" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ORD034</t>
+          <t>ORD033</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>IT132</t>
+          <t>IT125</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>9000</v>
+        <v>4000</v>
       </c>
       <c r="E91" t="n">
-        <v>27000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ORD034</t>
+          <t>ORD033</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>IT130</t>
+          <t>IT122</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D92" t="n">
-        <v>8500</v>
+        <v>3000</v>
       </c>
       <c r="E92" t="n">
-        <v>8500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ORD035</t>
+          <t>ORD034</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>IT149</t>
+          <t>IT139</t>
         </is>
       </c>
       <c r="C93" t="n">
         <v>3</v>
       </c>
       <c r="D93" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="E93" t="n">
-        <v>6000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ORD035</t>
+          <t>ORD034</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>IT147</t>
+          <t>IT140</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D94" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="E94" t="n">
-        <v>4500</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ORD036</t>
+          <t>ORD035</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IT163</t>
+          <t>IT148</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D95" t="n">
-        <v>19500</v>
+        <v>9000</v>
       </c>
       <c r="E95" t="n">
-        <v>19500</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ORD036</t>
+          <t>ORD035</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>IT158</t>
+          <t>IT146</t>
         </is>
       </c>
       <c r="C96" t="n">
         <v>3</v>
       </c>
       <c r="D96" t="n">
-        <v>8000</v>
+        <v>4000</v>
       </c>
       <c r="E96" t="n">
-        <v>24000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ORD036</t>
+          <t>ORD035</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IT159</t>
+          <t>IT144</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D97" t="n">
         <v>4500</v>
       </c>
       <c r="E97" t="n">
-        <v>9000</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ORD037</t>
+          <t>ORD036</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>IT012</t>
+          <t>IT157</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D98" t="n">
-        <v>5000</v>
+        <v>8500</v>
       </c>
       <c r="E98" t="n">
-        <v>10000</v>
+        <v>25500</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ORD037</t>
+          <t>ORD036</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>IT01</t>
+          <t>IT155</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D99" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="E99" t="n">
-        <v>5000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="100">
@@ -23555,38 +23349,38 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>IT174</t>
+          <t>IT009</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="E100" t="n">
-        <v>15000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ORD038</t>
+          <t>ORD037</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>IT186</t>
+          <t>IT033</t>
         </is>
       </c>
       <c r="C101" t="n">
         <v>2</v>
       </c>
       <c r="D101" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="E101" t="n">
-        <v>7000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="102">
@@ -23597,38 +23391,38 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>IT185</t>
+          <t>IT026</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D102" t="n">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="E102" t="n">
-        <v>12000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ORD039</t>
+          <t>ORD038</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>IT054</t>
+          <t>IT178</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D103" t="n">
-        <v>2500</v>
+        <v>5500</v>
       </c>
       <c r="E103" t="n">
-        <v>5000</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="104">
@@ -23639,101 +23433,101 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>IT056</t>
+          <t>IT050</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D104" t="n">
-        <v>1800</v>
+        <v>3500</v>
       </c>
       <c r="E104" t="n">
-        <v>1800</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ORD040</t>
+          <t>ORD039</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>IT058</t>
+          <t>IT054</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D105" t="n">
-        <v>6500</v>
+        <v>2500</v>
       </c>
       <c r="E105" t="n">
-        <v>6500</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ORD040</t>
+          <t>ORD039</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>IT200</t>
+          <t>IT194</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D106" t="n">
         <v>3000</v>
       </c>
       <c r="E106" t="n">
-        <v>9000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ORD041</t>
+          <t>ORD040</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>IT211</t>
+          <t>IT067</t>
         </is>
       </c>
       <c r="C107" t="n">
         <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>10000</v>
+        <v>3500</v>
       </c>
       <c r="E107" t="n">
-        <v>20000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ORD041</t>
+          <t>ORD040</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>IT072</t>
+          <t>IT065</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D108" t="n">
-        <v>7500</v>
+        <v>2500</v>
       </c>
       <c r="E108" t="n">
-        <v>7500</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="109">
@@ -23744,38 +23538,38 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>IT210</t>
+          <t>IT078</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D109" t="n">
-        <v>800</v>
+        <v>1300</v>
       </c>
       <c r="E109" t="n">
-        <v>800</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ORD042</t>
+          <t>ORD041</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>IT090</t>
+          <t>IT080</t>
         </is>
       </c>
       <c r="C110" t="n">
         <v>1</v>
       </c>
       <c r="D110" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="E110" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="111">
@@ -23786,17 +23580,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>IT218</t>
+          <t>IT091</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D111" t="n">
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="E111" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="112">
@@ -23807,38 +23601,38 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>IT216</t>
+          <t>IT218</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D112" t="n">
-        <v>6000</v>
+        <v>20000</v>
       </c>
       <c r="E112" t="n">
-        <v>18000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ORD043</t>
+          <t>ORD042</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>IT096</t>
+          <t>IT090</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D113" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="E113" t="n">
-        <v>30000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="114">
@@ -23849,122 +23643,185 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>IT102</t>
+          <t>IT096</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="E114" t="n">
-        <v>26000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>ORD044</t>
+          <t>ORD043</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>IT231</t>
+          <t>IT098</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>17500</v>
+        <v>7000</v>
       </c>
       <c r="E115" t="n">
-        <v>35000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ORD044</t>
+          <t>ORD043</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>IT107</t>
+          <t>IT225</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D116" t="n">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="E116" t="n">
-        <v>2000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ORD045</t>
+          <t>ORD044</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>IT125</t>
+          <t>IT105</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>4000</v>
+        <v>9500</v>
       </c>
       <c r="E117" t="n">
-        <v>8000</v>
+        <v>28500</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ORD045</t>
+          <t>ORD044</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>IT117</t>
+          <t>IT110</t>
         </is>
       </c>
       <c r="C118" t="n">
         <v>2</v>
       </c>
       <c r="D118" t="n">
-        <v>3500</v>
+        <v>6500</v>
       </c>
       <c r="E118" t="n">
-        <v>7000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
+          <t>ORD044</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>IT106</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
+      </c>
+      <c r="D119" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E119" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>ORD045</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>IT118</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>1</v>
-      </c>
-      <c r="D119" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E119" t="n">
-        <v>6000</v>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>IT117</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E120" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>ORD045</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>IT121</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>3</v>
+      </c>
+      <c r="D121" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E121" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ORD045</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>IT120</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E122" t="n">
+        <v>3500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add a service dashboard, and record when an order reached the table
</commit_message>
<xml_diff>
--- a/Chowly - Seed Data.xlsx
+++ b/Chowly - Seed Data.xlsx
@@ -908,12 +908,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-29 17:08</t>
+          <t>2026-08-30 17:08</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-29 17:52</t>
+          <t>2026-08-30 17:52</t>
         </is>
       </c>
     </row>
@@ -940,12 +940,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-29 12:06</t>
+          <t>2026-08-30 12:06</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 13:01</t>
+          <t>2026-08-30 13:01</t>
         </is>
       </c>
     </row>
@@ -972,12 +972,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-29 16:32</t>
+          <t>2026-08-30 16:32</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 17:23</t>
+          <t>2026-08-30 17:23</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-29 14:10</t>
+          <t>2026-08-30 14:10</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-29 14:59</t>
+          <t>2026-08-30 14:59</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1036,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-29 17:29</t>
+          <t>2026-08-30 17:29</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-29 17:58</t>
+          <t>2026-08-30 17:58</t>
         </is>
       </c>
     </row>
@@ -1068,12 +1068,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-30 20:19</t>
+          <t>2026-08-31 20:19</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-30 21:03</t>
+          <t>2026-08-31 21:03</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1100,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-30 14:53</t>
+          <t>2026-08-31 14:53</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-30 15:45</t>
+          <t>2026-08-31 15:45</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-30 15:04</t>
+          <t>2026-08-31 15:04</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-30 15:52</t>
+          <t>2026-08-31 15:52</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-30 16:08</t>
+          <t>2026-08-31 16:08</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-30 16:45</t>
+          <t>2026-08-31 16:45</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1196,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-30 19:53</t>
+          <t>2026-08-31 19:53</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-30 20:18</t>
+          <t>2026-08-31 20:18</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1228,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-31 16:41</t>
+          <t>2026-09-01 16:41</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-08-31 17:37</t>
+          <t>2026-09-01 17:37</t>
         </is>
       </c>
     </row>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-31 20:45</t>
+          <t>2026-09-01 20:45</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-31 21:03</t>
+          <t>2026-09-01 21:03</t>
         </is>
       </c>
     </row>
@@ -1284,12 +1284,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-31 20:38</t>
+          <t>2026-09-01 20:38</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-31 20:59</t>
+          <t>2026-09-01 20:59</t>
         </is>
       </c>
     </row>
@@ -1312,12 +1312,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-31 13:25</t>
+          <t>2026-09-01 13:25</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-31 14:16</t>
+          <t>2026-09-01 14:16</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-06 23:24</t>
+          <t>2026-09-07 08:47</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-06 23:26</t>
+          <t>2026-09-07 08:49</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1400,12 +1400,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-01 16:05</t>
+          <t>2026-09-02 16:05</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-01 16:16</t>
+          <t>2026-09-02 16:16</t>
         </is>
       </c>
     </row>
@@ -1432,12 +1432,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-01 18:19</t>
+          <t>2026-09-02 18:19</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-01 19:00</t>
+          <t>2026-09-02 19:00</t>
         </is>
       </c>
     </row>
@@ -1464,12 +1464,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-01 17:24</t>
+          <t>2026-09-02 17:24</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-01 18:12</t>
+          <t>2026-09-02 18:12</t>
         </is>
       </c>
     </row>
@@ -1496,12 +1496,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-01 20:34</t>
+          <t>2026-09-02 20:34</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-01 21:21</t>
+          <t>2026-09-02 21:21</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1528,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-01 19:08</t>
+          <t>2026-09-02 19:08</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-01 20:13</t>
+          <t>2026-09-02 20:13</t>
         </is>
       </c>
     </row>
@@ -1560,12 +1560,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-02 15:39</t>
+          <t>2026-09-03 15:39</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-02 15:53</t>
+          <t>2026-09-03 15:53</t>
         </is>
       </c>
     </row>
@@ -1592,12 +1592,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-02 16:33</t>
+          <t>2026-09-03 16:33</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-02 17:42</t>
+          <t>2026-09-03 17:42</t>
         </is>
       </c>
     </row>
@@ -1620,12 +1620,12 @@
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-02 16:59</t>
+          <t>2026-09-03 16:59</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-02 17:29</t>
+          <t>2026-09-03 17:29</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-06 23:15</t>
+          <t>2026-09-07 08:38</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-06 23:45</t>
+          <t>2026-09-07 09:08</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1704,12 +1704,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-02 15:06</t>
+          <t>2026-09-03 15:06</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-02 16:22</t>
+          <t>2026-09-03 16:22</t>
         </is>
       </c>
     </row>
@@ -1736,12 +1736,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-03 14:03</t>
+          <t>2026-09-04 14:03</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-03 14:24</t>
+          <t>2026-09-04 14:24</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-03 20:15</t>
+          <t>2026-09-04 20:15</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-03 20:40</t>
+          <t>2026-09-04 20:40</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1796,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-03 16:55</t>
+          <t>2026-09-04 16:55</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-03 17:13</t>
+          <t>2026-09-04 17:13</t>
         </is>
       </c>
     </row>
@@ -1824,12 +1824,12 @@
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-03 19:09</t>
+          <t>2026-09-04 19:09</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-03 20:13</t>
+          <t>2026-09-04 20:13</t>
         </is>
       </c>
     </row>
@@ -1852,12 +1852,12 @@
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-03 15:05</t>
+          <t>2026-09-04 15:05</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-03 15:50</t>
+          <t>2026-09-04 15:50</t>
         </is>
       </c>
     </row>
@@ -1884,12 +1884,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-04 17:29</t>
+          <t>2026-09-05 17:29</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-04 18:21</t>
+          <t>2026-09-05 18:21</t>
         </is>
       </c>
     </row>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-04 13:50</t>
+          <t>2026-09-05 13:50</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-09-04 14:49</t>
+          <t>2026-09-05 14:49</t>
         </is>
       </c>
     </row>
@@ -1948,12 +1948,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-04 20:49</t>
+          <t>2026-09-05 20:49</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-04 21:05</t>
+          <t>2026-09-05 21:05</t>
         </is>
       </c>
     </row>
@@ -1976,12 +1976,12 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-04 16:11</t>
+          <t>2026-09-05 16:11</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-04 16:25</t>
+          <t>2026-09-05 16:25</t>
         </is>
       </c>
     </row>
@@ -2004,12 +2004,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-04 19:54</t>
+          <t>2026-09-05 19:54</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-09-04 20:39</t>
+          <t>2026-09-05 20:39</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-06 23:37</t>
+          <t>2026-09-07 09:00</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2060,12 +2060,12 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-05 13:38</t>
+          <t>2026-09-06 13:38</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-09-05 14:45</t>
+          <t>2026-09-06 14:45</t>
         </is>
       </c>
     </row>
@@ -2088,12 +2088,12 @@
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-05 19:22</t>
+          <t>2026-09-06 19:22</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-09-05 20:24</t>
+          <t>2026-09-06 20:24</t>
         </is>
       </c>
     </row>
@@ -2116,12 +2116,12 @@
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-05 17:46</t>
+          <t>2026-09-06 17:46</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-05 18:16</t>
+          <t>2026-09-06 18:16</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-29 17:57</t>
+          <t>2026-08-30 17:57</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-29 13:04</t>
+          <t>2026-08-30 13:04</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-29 17:24</t>
+          <t>2026-08-30 17:24</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-29 15:05</t>
+          <t>2026-08-30 15:05</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-29 18:01</t>
+          <t>2026-08-30 18:01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-30 15:49</t>
+          <t>2026-08-31 15:49</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-30 15:58</t>
+          <t>2026-08-31 15:58</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-30 16:48</t>
+          <t>2026-08-31 16:48</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-31 14:19</t>
+          <t>2026-09-01 14:19</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-01 19:05</t>
+          <t>2026-09-02 19:05</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-01 18:17</t>
+          <t>2026-09-02 18:17</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-01 21:23</t>
+          <t>2026-09-02 21:23</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-01 20:18</t>
+          <t>2026-09-02 20:18</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-02 17:46</t>
+          <t>2026-09-03 17:46</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-02 16:26</t>
+          <t>2026-09-03 16:26</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2703,7 +2703,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-03 20:44</t>
+          <t>2026-09-04 20:44</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-03 20:18</t>
+          <t>2026-09-04 20:18</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2767,7 +2767,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-04 18:26</t>
+          <t>2026-09-05 18:26</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-04 14:54</t>
+          <t>2026-09-05 14:54</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-04 20:42</t>
+          <t>2026-09-05 20:42</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-05 14:46</t>
+          <t>2026-09-06 14:46</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-05 20:26</t>
+          <t>2026-09-06 20:26</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-29 18:02</t>
+          <t>2026-08-30 18:02</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3035,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 13:09</t>
+          <t>2026-08-30 13:09</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 17:32</t>
+          <t>2026-08-30 17:32</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-29 15:07</t>
+          <t>2026-08-30 15:07</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-29 18:03</t>
+          <t>2026-08-30 18:03</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-30 21:06</t>
+          <t>2026-08-31 21:06</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3185,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-30 15:52</t>
+          <t>2026-08-31 15:52</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-30 15:54</t>
+          <t>2026-08-31 15:54</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3245,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-30 16:54</t>
+          <t>2026-08-31 16:54</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-30 20:21</t>
+          <t>2026-08-31 20:21</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-08-31 17:44</t>
+          <t>2026-09-01 17:44</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-08-31 21:10</t>
+          <t>2026-09-01 21:10</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-08-31 21:03</t>
+          <t>2026-09-01 21:03</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3395,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-08-31 14:26</t>
+          <t>2026-09-01 14:26</t>
         </is>
       </c>
     </row>
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-01 16:26</t>
+          <t>2026-09-02 16:26</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3455,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-09-01 19:03</t>
+          <t>2026-09-02 19:03</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-01 18:14</t>
+          <t>2026-09-02 18:14</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-09-01 21:30</t>
+          <t>2026-09-02 21:30</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-09-01 20:16</t>
+          <t>2026-09-02 20:16</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-02 15:57</t>
+          <t>2026-09-03 15:57</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-09-02 17:49</t>
+          <t>2026-09-03 17:49</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-02 17:37</t>
+          <t>2026-09-03 17:37</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-09-02 16:24</t>
+          <t>2026-09-03 16:24</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-03 14:30</t>
+          <t>2026-09-04 14:30</t>
         </is>
       </c>
     </row>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-03 20:46</t>
+          <t>2026-09-04 20:46</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-03 17:20</t>
+          <t>2026-09-04 17:20</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-09-03 20:16</t>
+          <t>2026-09-04 20:16</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-03 15:52</t>
+          <t>2026-09-04 15:52</t>
         </is>
       </c>
     </row>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-04 18:23</t>
+          <t>2026-09-05 18:23</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-04 14:51</t>
+          <t>2026-09-05 14:51</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-09-04 20:47</t>
+          <t>2026-09-05 20:47</t>
         </is>
       </c>
     </row>
@@ -3935,7 +3935,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-05 14:51</t>
+          <t>2026-09-06 14:51</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3965,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-09-05 20:33</t>
+          <t>2026-09-06 20:33</t>
         </is>
       </c>
     </row>
@@ -4076,12 +4076,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>CHW-20260829-0001</t>
+          <t>CHW-20260830-0001</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-08-29 17:57</t>
+          <t>2026-08-30 17:57</t>
         </is>
       </c>
     </row>
@@ -4111,12 +4111,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>CHW-20260829-0002</t>
+          <t>CHW-20260830-0002</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-08-29 13:11</t>
+          <t>2026-08-30 13:11</t>
         </is>
       </c>
     </row>
@@ -4146,12 +4146,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>CHW-20260829-0003</t>
+          <t>CHW-20260830-0003</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-08-29 17:39</t>
+          <t>2026-08-30 17:39</t>
         </is>
       </c>
     </row>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>CHW-20260829-0004</t>
+          <t>CHW-20260830-0004</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-08-29 15:18</t>
+          <t>2026-08-30 15:18</t>
         </is>
       </c>
     </row>
@@ -4216,12 +4216,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>CHW-20260829-0005</t>
+          <t>CHW-20260830-0005</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-08-29 18:16</t>
+          <t>2026-08-30 18:16</t>
         </is>
       </c>
     </row>
@@ -4251,12 +4251,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>CHW-20260829-0006</t>
+          <t>CHW-20260830-0006</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-30 15:59</t>
+          <t>2026-08-31 15:59</t>
         </is>
       </c>
     </row>
@@ -4286,12 +4286,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>CHW-20260829-0007</t>
+          <t>CHW-20260830-0007</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-30 16:10</t>
+          <t>2026-08-31 16:10</t>
         </is>
       </c>
     </row>
@@ -4321,12 +4321,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>CHW-20260829-0008</t>
+          <t>CHW-20260830-0008</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-30 17:01</t>
+          <t>2026-08-31 17:01</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4356,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>CHW-20260829-0009</t>
+          <t>CHW-20260830-0009</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-30 20:34</t>
+          <t>2026-08-31 20:34</t>
         </is>
       </c>
     </row>
@@ -4391,12 +4391,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>CHW-20260829-0010</t>
+          <t>CHW-20260830-0010</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-08-31 17:42</t>
+          <t>2026-09-01 17:42</t>
         </is>
       </c>
     </row>
@@ -4426,12 +4426,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>CHW-20260829-0011</t>
+          <t>CHW-20260830-0011</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-08-31 21:14</t>
+          <t>2026-09-01 21:14</t>
         </is>
       </c>
     </row>
@@ -4461,12 +4461,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>CHW-20260829-0012</t>
+          <t>CHW-20260830-0012</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-08-31 14:35</t>
+          <t>2026-09-01 14:35</t>
         </is>
       </c>
     </row>
@@ -4496,12 +4496,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>CHW-20260829-0013</t>
+          <t>CHW-20260830-0013</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-01 16:32</t>
+          <t>2026-09-02 16:32</t>
         </is>
       </c>
     </row>
@@ -4531,12 +4531,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CHW-20260829-0014</t>
+          <t>CHW-20260830-0014</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-09-01 18:22</t>
+          <t>2026-09-02 18:22</t>
         </is>
       </c>
     </row>
@@ -4566,12 +4566,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CHW-20260829-0015</t>
+          <t>CHW-20260830-0015</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-09-01 21:29</t>
+          <t>2026-09-02 21:29</t>
         </is>
       </c>
     </row>
@@ -4601,12 +4601,12 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CHW-20260829-0016</t>
+          <t>CHW-20260830-0016</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-09-01 20:16</t>
+          <t>2026-09-02 20:16</t>
         </is>
       </c>
     </row>
@@ -4636,12 +4636,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>CHW-20260829-0017</t>
+          <t>CHW-20260830-0017</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-02 16:01</t>
+          <t>2026-09-03 16:01</t>
         </is>
       </c>
     </row>
@@ -4671,12 +4671,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CHW-20260829-0018</t>
+          <t>CHW-20260830-0018</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-09-02 17:51</t>
+          <t>2026-09-03 17:51</t>
         </is>
       </c>
     </row>
@@ -4706,12 +4706,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>CHW-20260829-0019</t>
+          <t>CHW-20260830-0019</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-09-02 17:33</t>
+          <t>2026-09-03 17:33</t>
         </is>
       </c>
     </row>
@@ -4741,12 +4741,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>CHW-20260829-0020</t>
+          <t>CHW-20260830-0020</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-09-03 14:27</t>
+          <t>2026-09-04 14:27</t>
         </is>
       </c>
     </row>
@@ -4776,12 +4776,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>CHW-20260829-0021</t>
+          <t>CHW-20260830-0021</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-09-03 21:00</t>
+          <t>2026-09-04 21:00</t>
         </is>
       </c>
     </row>
@@ -4811,12 +4811,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>CHW-20260829-0022</t>
+          <t>CHW-20260830-0022</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-09-03 20:30</t>
+          <t>2026-09-04 20:30</t>
         </is>
       </c>
     </row>
@@ -4846,12 +4846,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>CHW-20260829-0023</t>
+          <t>CHW-20260830-0023</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-09-03 15:53</t>
+          <t>2026-09-04 15:53</t>
         </is>
       </c>
     </row>
@@ -4881,12 +4881,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CHW-20260829-0024</t>
+          <t>CHW-20260830-0024</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-09-04 15:09</t>
+          <t>2026-09-05 15:09</t>
         </is>
       </c>
     </row>
@@ -4916,12 +4916,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>CHW-20260829-0025</t>
+          <t>CHW-20260830-0025</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-09-04 21:19</t>
+          <t>2026-09-05 21:19</t>
         </is>
       </c>
     </row>
@@ -4951,12 +4951,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>CHW-20260829-0026</t>
+          <t>CHW-20260830-0026</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-09-04 16:45</t>
+          <t>2026-09-05 16:45</t>
         </is>
       </c>
     </row>
@@ -4986,12 +4986,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>CHW-20260829-0027</t>
+          <t>CHW-20260830-0027</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-09-04 20:43</t>
+          <t>2026-09-05 20:43</t>
         </is>
       </c>
     </row>
@@ -5021,12 +5021,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>CHW-20260829-0028</t>
+          <t>CHW-20260830-0028</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-09-05 14:52</t>
+          <t>2026-09-06 14:52</t>
         </is>
       </c>
     </row>
@@ -5056,12 +5056,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>CHW-20260829-0029</t>
+          <t>CHW-20260830-0029</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-09-05 20:28</t>
+          <t>2026-09-06 20:28</t>
         </is>
       </c>
     </row>
@@ -5091,12 +5091,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>CHW-20260829-0030</t>
+          <t>CHW-20260830-0030</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-09-05 18:21</t>
+          <t>2026-09-06 18:21</t>
         </is>
       </c>
     </row>
@@ -19371,7 +19371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19383,6 +19383,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19452,6 +19453,11 @@
           <t>table_number</t>
         </is>
       </c>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>served_at</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -19476,7 +19482,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-29 17:05</t>
+          <t>2026-08-30 17:05</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -19493,6 +19499,11 @@
       <c r="I6" t="n">
         <v>14</v>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:52</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -19517,7 +19528,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-06 23:15</t>
+          <t>2026-09-07 08:38</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -19534,6 +19545,7 @@
       <c r="I7" t="n">
         <v>5</v>
       </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19558,7 +19570,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-29 12:03</t>
+          <t>2026-08-30 12:03</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -19575,6 +19587,11 @@
       <c r="I8" t="n">
         <v>1</v>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-08-30 13:01</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -19599,7 +19616,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-29 16:31</t>
+          <t>2026-08-30 16:31</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -19616,6 +19633,11 @@
       <c r="I9" t="n">
         <v>20</v>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:23</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -19640,7 +19662,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-29 14:06</t>
+          <t>2026-08-30 14:06</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -19657,6 +19679,11 @@
       <c r="I10" t="n">
         <v>13</v>
       </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-08-30 14:59</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -19681,7 +19708,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-29 17:27</t>
+          <t>2026-08-30 17:27</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -19698,6 +19725,11 @@
       <c r="I11" t="n">
         <v>13</v>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:58</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19722,7 +19754,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-30 20:16</t>
+          <t>2026-08-31 20:16</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -19739,6 +19771,11 @@
       <c r="I12" t="n">
         <v>11</v>
       </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-08-31 21:03</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19763,7 +19800,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-30 14:50</t>
+          <t>2026-08-31 14:50</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -19780,6 +19817,11 @@
       <c r="I13" t="n">
         <v>9</v>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-08-31 15:45</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19804,7 +19846,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-30 15:01</t>
+          <t>2026-08-31 15:01</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -19821,6 +19863,11 @@
       <c r="I14" t="n">
         <v>6</v>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-08-31 15:52</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -19845,7 +19892,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-06 23:32</t>
+          <t>2026-09-07 08:55</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -19862,6 +19909,7 @@
       <c r="I15" t="n">
         <v>17</v>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -19886,7 +19934,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-30 16:05</t>
+          <t>2026-08-31 16:05</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -19903,6 +19951,11 @@
       <c r="I16" t="n">
         <v>16</v>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-08-31 16:45</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -19927,7 +19980,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-30 19:49</t>
+          <t>2026-08-31 19:49</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -19944,6 +19997,11 @@
       <c r="I17" t="n">
         <v>1</v>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-08-31 20:18</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -19968,7 +20026,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-08-31 16:38</t>
+          <t>2026-09-01 16:38</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -19985,6 +20043,11 @@
       <c r="I18" t="n">
         <v>16</v>
       </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-09-01 17:37</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -20009,7 +20072,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-08-31 20:43</t>
+          <t>2026-09-01 20:43</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -20026,6 +20089,11 @@
       <c r="I19" t="n">
         <v>6</v>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-09-01 21:03</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -20050,7 +20118,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-08-31 20:37</t>
+          <t>2026-09-01 20:37</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -20067,6 +20135,11 @@
       <c r="I20" t="n">
         <v>5</v>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-09-01 20:59</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -20091,7 +20164,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-06 23:43</t>
+          <t>2026-09-07 09:06</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -20108,6 +20181,7 @@
       <c r="I21" t="n">
         <v>19</v>
       </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -20132,7 +20206,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-31 13:23</t>
+          <t>2026-09-01 13:23</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -20149,6 +20223,11 @@
       <c r="I22" t="n">
         <v>22</v>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-09-01 14:16</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -20173,7 +20252,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-06 23:22</t>
+          <t>2026-09-07 08:45</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -20190,6 +20269,7 @@
       <c r="I23" t="n">
         <v>16</v>
       </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -20214,7 +20294,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-06 23:24</t>
+          <t>2026-09-07 08:47</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -20231,6 +20311,7 @@
       <c r="I24" t="n">
         <v>4</v>
       </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -20255,7 +20336,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-01 16:01</t>
+          <t>2026-09-02 16:01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -20272,6 +20353,11 @@
       <c r="I25" t="n">
         <v>1</v>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-09-02 16:16</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -20296,7 +20382,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-01 18:16</t>
+          <t>2026-09-02 18:16</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -20313,6 +20399,11 @@
       <c r="I26" t="n">
         <v>5</v>
       </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-09-02 19:00</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -20337,7 +20428,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-01 17:20</t>
+          <t>2026-09-02 17:20</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -20354,6 +20445,11 @@
       <c r="I27" t="n">
         <v>17</v>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-09-02 18:12</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -20378,7 +20474,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-01 20:30</t>
+          <t>2026-09-02 20:30</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -20395,6 +20491,11 @@
       <c r="I28" t="n">
         <v>5</v>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-09-02 21:21</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -20419,7 +20520,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-01 19:05</t>
+          <t>2026-09-02 19:05</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -20436,6 +20537,11 @@
       <c r="I29" t="n">
         <v>6</v>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-09-02 20:13</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -20460,7 +20566,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-02 15:35</t>
+          <t>2026-09-03 15:35</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -20477,6 +20583,11 @@
       <c r="I30" t="n">
         <v>11</v>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-09-03 15:53</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -20501,7 +20612,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-02 16:30</t>
+          <t>2026-09-03 16:30</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -20518,6 +20629,11 @@
       <c r="I31" t="n">
         <v>4</v>
       </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:42</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -20542,7 +20658,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-02 16:58</t>
+          <t>2026-09-03 16:58</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -20559,6 +20675,11 @@
       <c r="I32" t="n">
         <v>6</v>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-09-03 17:29</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -20583,7 +20704,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-06 23:11</t>
+          <t>2026-09-07 08:34</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -20600,6 +20721,7 @@
       <c r="I33" t="n">
         <v>23</v>
       </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -20624,7 +20746,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-06 23:42</t>
+          <t>2026-09-07 09:05</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -20641,6 +20763,7 @@
       <c r="I34" t="n">
         <v>8</v>
       </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -20665,7 +20788,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-02 15:02</t>
+          <t>2026-09-03 15:02</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -20682,6 +20805,11 @@
       <c r="I35" t="n">
         <v>23</v>
       </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-09-03 16:22</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -20706,7 +20834,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-03 14:02</t>
+          <t>2026-09-04 14:02</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -20723,6 +20851,11 @@
       <c r="I36" t="n">
         <v>19</v>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-09-04 14:24</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -20747,7 +20880,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-06 23:33</t>
+          <t>2026-09-07 08:56</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -20764,6 +20897,7 @@
       <c r="I37" t="n">
         <v>22</v>
       </c>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20788,7 +20922,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-03 20:13</t>
+          <t>2026-09-04 20:13</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -20805,6 +20939,11 @@
       <c r="I38" t="n">
         <v>21</v>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-09-04 20:40</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -20829,7 +20968,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-03 16:54</t>
+          <t>2026-09-04 16:54</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -20846,6 +20985,11 @@
       <c r="I39" t="n">
         <v>8</v>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-09-04 17:13</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -20870,7 +21014,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-03 19:08</t>
+          <t>2026-09-04 19:08</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -20887,6 +21031,11 @@
       <c r="I40" t="n">
         <v>15</v>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-09-04 20:13</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -20911,7 +21060,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-03 15:04</t>
+          <t>2026-09-04 15:04</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -20928,6 +21077,11 @@
       <c r="I41" t="n">
         <v>2</v>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-09-04 15:50</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -20952,7 +21106,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-04 17:25</t>
+          <t>2026-09-05 17:25</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -20969,6 +21123,11 @@
       <c r="I42" t="n">
         <v>9</v>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-09-05 18:21</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -20993,7 +21152,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-04 13:49</t>
+          <t>2026-09-05 13:49</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -21010,6 +21169,11 @@
       <c r="I43" t="n">
         <v>11</v>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-09-05 14:49</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -21034,7 +21198,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-04 20:48</t>
+          <t>2026-09-05 20:48</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -21051,6 +21215,11 @@
       <c r="I44" t="n">
         <v>1</v>
       </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-09-05 21:05</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -21075,7 +21244,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-04 16:09</t>
+          <t>2026-09-05 16:09</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -21092,6 +21261,11 @@
       <c r="I45" t="n">
         <v>11</v>
       </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-09-05 16:25</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -21116,7 +21290,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-04 19:52</t>
+          <t>2026-09-05 19:52</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -21133,6 +21307,11 @@
       <c r="I46" t="n">
         <v>6</v>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-09-05 20:39</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -21157,7 +21336,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-06 23:33</t>
+          <t>2026-09-07 08:56</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21174,6 +21353,7 @@
       <c r="I47" t="n">
         <v>17</v>
       </c>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -21198,7 +21378,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-05 13:35</t>
+          <t>2026-09-06 13:35</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -21215,6 +21395,11 @@
       <c r="I48" t="n">
         <v>11</v>
       </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-09-06 14:45</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -21239,7 +21424,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-09-05 19:18</t>
+          <t>2026-09-06 19:18</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -21256,6 +21441,11 @@
       <c r="I49" t="n">
         <v>22</v>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-09-06 20:24</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -21280,7 +21470,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-09-05 17:44</t>
+          <t>2026-09-06 17:44</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -21296,6 +21486,11 @@
       </c>
       <c r="I50" t="n">
         <v>12</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:16</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebuild seeded orders instead of upserting them
</commit_message>
<xml_diff>
--- a/Chowly - Seed Data.xlsx
+++ b/Chowly - Seed Data.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>655</v>
+        <v>656</v>
       </c>
     </row>
     <row r="19">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-31 21:03</t>
+          <t>2026-08-31 20:58</t>
         </is>
       </c>
     </row>
@@ -1093,19 +1093,15 @@
           <t>S231</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>S232</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-31 14:53</t>
+          <t>2026-08-31 18:52</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-31 15:45</t>
+          <t>2026-08-31 20:03</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1128,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-31 15:04</t>
+          <t>2026-08-31 18:48</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-31 15:52</t>
+          <t>2026-08-31 19:26</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1160,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-31 16:08</t>
+          <t>2026-08-31 16:22</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-31 16:45</t>
+          <t>2026-08-31 17:25</t>
         </is>
       </c>
     </row>
@@ -1196,12 +1192,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-08-31 19:53</t>
+          <t>2026-08-31 13:57</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-31 20:18</t>
+          <t>2026-08-31 14:23</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1224,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-01 16:41</t>
+          <t>2026-09-01 17:20</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-01 17:37</t>
+          <t>2026-09-01 18:11</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1257,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-01 21:03</t>
+          <t>2026-09-01 20:58</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1285,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-01 20:59</t>
+          <t>2026-09-01 20:54</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1340,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-07 08:47</t>
+          <t>2026-09-07 09:16</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1372,7 +1368,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-07 08:49</t>
+          <t>2026-09-07 09:18</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1405,7 +1401,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-09-02 16:16</t>
+          <t>2026-09-02 16:11</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1561,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-03 15:53</t>
+          <t>2026-09-03 15:48</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1621,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-03 17:29</t>
+          <t>2026-09-03 17:24</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1644,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-07 08:38</t>
+          <t>2026-09-07 09:07</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1676,7 +1672,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-07 09:08</t>
+          <t>2026-09-07 09:37</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -1741,7 +1737,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-04 14:24</t>
+          <t>2026-09-04 14:19</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1764,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-04 20:15</t>
+          <t>2026-09-04 12:04</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-09-04 20:40</t>
+          <t>2026-09-04 12:54</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1784,11 @@
           <t>ORD034</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>S239</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>S240</t>
@@ -1796,12 +1796,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-04 16:55</t>
+          <t>2026-09-04 16:18</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-09-04 17:13</t>
+          <t>2026-09-04 16:37</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1857,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-09-04 15:50</t>
+          <t>2026-09-04 15:45</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-09-05 21:05</t>
+          <t>2026-09-05 21:00</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-09-05 16:25</t>
+          <t>2026-09-05 16:20</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-07 09:00</t>
+          <t>2026-09-07 09:29</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -2121,7 +2121,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-09-06 18:16</t>
+          <t>2026-09-06 18:11</t>
         </is>
       </c>
     </row>
@@ -2373,17 +2373,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>C011</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Order took far longer than the quoted time</t>
+          <t>Drinks came very late</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-31 15:49</t>
+          <t>2026-08-31 20:04</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -2405,17 +2405,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>C013</t>
+          <t>C012</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Drinks came very late</t>
+          <t>We waited well past the estimated wait</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-31 15:58</t>
+          <t>2026-08-31 19:30</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2437,17 +2437,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>C009</t>
+          <t>C004</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Order took far longer than the quoted time</t>
+          <t>Serious delay before the food arrived</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-31 16:48</t>
+          <t>2026-08-31 17:26</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2693,22 +2693,22 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>We waited well past the estimated wait</t>
+          <t>Serious delay before the food arrived</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-04 20:44</t>
+          <t>2026-09-04 12:55</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -3150,12 +3150,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Excellent service</t>
+          <t>Will come again</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-31 21:06</t>
+          <t>2026-08-31 21:00</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>C011</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-31 15:52</t>
+          <t>2026-08-31 20:11</t>
         </is>
       </c>
     </row>
@@ -3202,11 +3202,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>C013</t>
+          <t>C012</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-31 15:54</t>
+          <t>2026-08-31 19:32</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>C009</t>
+          <t>C004</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -3240,12 +3240,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Long waiting time</t>
+          <t>Not happy with the delay</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-31 16:54</t>
+          <t>2026-08-31 17:28</t>
         </is>
       </c>
     </row>
@@ -3262,20 +3262,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Lovely food</t>
+          <t>Very good</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-31 20:21</t>
+          <t>2026-08-31 14:28</t>
         </is>
       </c>
     </row>
@@ -3292,11 +3292,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>C019</t>
+          <t>C021</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-09-01 17:44</t>
+          <t>2026-09-01 18:18</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-09-01 21:10</t>
+          <t>2026-09-01 21:05</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-09-01 21:03</t>
+          <t>2026-09-01 20:58</t>
         </is>
       </c>
     </row>
@@ -3416,7 +3416,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3425,7 +3425,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-09-02 16:26</t>
+          <t>2026-09-02 16:21</t>
         </is>
       </c>
     </row>
@@ -3566,7 +3566,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-09-03 15:57</t>
+          <t>2026-09-03 15:52</t>
         </is>
       </c>
     </row>
@@ -3626,7 +3626,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-09-03 17:37</t>
+          <t>2026-09-03 17:32</t>
         </is>
       </c>
     </row>
@@ -3686,16 +3686,16 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Excellent service</t>
+          <t>Lovely food</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-09-04 14:30</t>
+          <t>2026-09-04 14:29</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3712,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -3720,12 +3720,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Long waiting time</t>
+          <t>Not happy with the delay</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-09-04 20:46</t>
+          <t>2026-09-04 13:02</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>C009</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-09-04 17:20</t>
+          <t>2026-09-04 16:44</t>
         </is>
       </c>
     </row>
@@ -3806,16 +3806,16 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Excellent service</t>
+          <t>Lovely food</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-09-04 15:52</t>
+          <t>2026-09-04 15:47</t>
         </is>
       </c>
     </row>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>16500</v>
+        <v>19000</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-08-31 15:59</t>
+          <t>2026-08-31 20:17</t>
         </is>
       </c>
     </row>
@@ -4272,11 +4272,11 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>18900</v>
+        <v>15000</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Card</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4291,7 +4291,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-08-31 16:10</t>
+          <t>2026-08-31 19:41</t>
         </is>
       </c>
     </row>
@@ -4307,11 +4307,11 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>16500</v>
+        <v>23500</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Card</t>
+          <t>Bank Transfer</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-08-31 17:01</t>
+          <t>2026-08-31 17:33</t>
         </is>
       </c>
     </row>
@@ -4342,7 +4342,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>28000</v>
+        <v>37500</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-08-31 20:34</t>
+          <t>2026-08-31 14:33</t>
         </is>
       </c>
     </row>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-09-01 17:42</t>
+          <t>2026-09-01 18:16</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-09-01 21:14</t>
+          <t>2026-09-01 21:09</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-09-02 16:32</t>
+          <t>2026-09-02 16:27</t>
         </is>
       </c>
     </row>
@@ -4641,7 +4641,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-09-03 16:01</t>
+          <t>2026-09-03 15:56</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-09-03 17:33</t>
+          <t>2026-09-03 17:28</t>
         </is>
       </c>
     </row>
@@ -4746,7 +4746,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-09-04 14:27</t>
+          <t>2026-09-04 14:24</t>
         </is>
       </c>
     </row>
@@ -4762,11 +4762,11 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>10000</v>
+        <v>15500</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Bank Transfer</t>
+          <t>Card</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-09-04 21:00</t>
+          <t>2026-09-04 13:14</t>
         </is>
       </c>
     </row>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>Card</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -4851,7 +4851,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-09-04 15:53</t>
+          <t>2026-09-04 15:48</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-09-05 21:19</t>
+          <t>2026-09-05 21:14</t>
         </is>
       </c>
     </row>
@@ -4956,7 +4956,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-09-05 16:45</t>
+          <t>2026-09-05 16:40</t>
         </is>
       </c>
     </row>
@@ -5096,7 +5096,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-09-06 18:21</t>
+          <t>2026-09-06 18:16</t>
         </is>
       </c>
     </row>
@@ -19528,7 +19528,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-07 08:38</t>
+          <t>2026-09-07 09:07</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -19773,7 +19773,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-31 21:03</t>
+          <t>2026-08-31 20:58</t>
         </is>
       </c>
     </row>
@@ -19785,7 +19785,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C011</t>
+          <t>C003</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -19800,7 +19800,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-08-31 14:50</t>
+          <t>2026-08-31 18:49</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -19809,17 +19809,17 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H13" t="n">
-        <v>16500</v>
+        <v>19000</v>
       </c>
       <c r="I13" t="n">
         <v>9</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-31 15:45</t>
+          <t>2026-08-31 20:03</t>
         </is>
       </c>
     </row>
@@ -19831,7 +19831,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>C013</t>
+          <t>C012</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -19846,7 +19846,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-08-31 15:01</t>
+          <t>2026-08-31 18:45</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -19855,17 +19855,17 @@
         </is>
       </c>
       <c r="G14" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H14" t="n">
-        <v>18900</v>
+        <v>15000</v>
       </c>
       <c r="I14" t="n">
         <v>6</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-31 15:52</t>
+          <t>2026-08-31 19:26</t>
         </is>
       </c>
     </row>
@@ -19877,7 +19877,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>C014</t>
+          <t>C019</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -19887,12 +19887,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>S241</t>
+          <t>S238</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-07 08:55</t>
+          <t>2026-09-07 09:09</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -19901,10 +19901,10 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="H15" t="n">
-        <v>9000</v>
+        <v>36500</v>
       </c>
       <c r="I15" t="n">
         <v>17</v>
@@ -19919,7 +19919,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>C009</t>
+          <t>C004</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -19929,12 +19929,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>S245</t>
+          <t>S242</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-08-31 16:05</t>
+          <t>2026-08-31 16:18</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -19943,17 +19943,17 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="H16" t="n">
-        <v>16500</v>
+        <v>23500</v>
       </c>
       <c r="I16" t="n">
         <v>16</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-31 16:45</t>
+          <t>2026-08-31 17:25</t>
         </is>
       </c>
     </row>
@@ -19965,7 +19965,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -19980,7 +19980,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-08-31 19:49</t>
+          <t>2026-08-31 13:56</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -19992,14 +19992,14 @@
         <v>28</v>
       </c>
       <c r="H17" t="n">
-        <v>28000</v>
+        <v>37500</v>
       </c>
       <c r="I17" t="n">
         <v>1</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-31 20:18</t>
+          <t>2026-08-31 14:23</t>
         </is>
       </c>
     </row>
@@ -20011,7 +20011,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>C019</t>
+          <t>C021</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -20026,7 +20026,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-01 16:38</t>
+          <t>2026-09-01 17:17</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -20045,7 +20045,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-01 17:37</t>
+          <t>2026-09-01 18:11</t>
         </is>
       </c>
     </row>
@@ -20091,7 +20091,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-01 21:03</t>
+          <t>2026-09-01 20:58</t>
         </is>
       </c>
     </row>
@@ -20137,7 +20137,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-01 20:59</t>
+          <t>2026-09-01 20:54</t>
         </is>
       </c>
     </row>
@@ -20164,7 +20164,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-07 09:06</t>
+          <t>2026-09-07 09:35</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -20252,7 +20252,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-07 08:45</t>
+          <t>2026-09-07 09:14</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -20294,7 +20294,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-07 08:47</t>
+          <t>2026-09-07 09:16</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -20355,7 +20355,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-02 16:16</t>
+          <t>2026-09-02 16:11</t>
         </is>
       </c>
     </row>
@@ -20585,7 +20585,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-03 15:53</t>
+          <t>2026-09-03 15:48</t>
         </is>
       </c>
     </row>
@@ -20677,7 +20677,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-03 17:29</t>
+          <t>2026-09-03 17:24</t>
         </is>
       </c>
     </row>
@@ -20704,7 +20704,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-07 08:34</t>
+          <t>2026-09-07 09:03</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -20746,7 +20746,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-07 09:05</t>
+          <t>2026-09-07 09:34</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -20853,7 +20853,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-04 14:24</t>
+          <t>2026-09-04 14:19</t>
         </is>
       </c>
     </row>
@@ -20865,7 +20865,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>C009</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-07 08:56</t>
+          <t>2026-09-07 09:40</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -20892,7 +20892,7 @@
         <v>13</v>
       </c>
       <c r="H37" t="n">
-        <v>10000</v>
+        <v>38000</v>
       </c>
       <c r="I37" t="n">
         <v>22</v>
@@ -20907,7 +20907,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C014</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -20917,12 +20917,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>S234</t>
+          <t>S237</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-04 20:13</t>
+          <t>2026-09-04 12:01</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -20934,14 +20934,14 @@
         <v>11</v>
       </c>
       <c r="H38" t="n">
-        <v>10000</v>
+        <v>15500</v>
       </c>
       <c r="I38" t="n">
         <v>21</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-09-04 20:40</t>
+          <t>2026-09-04 12:54</t>
         </is>
       </c>
     </row>
@@ -20953,7 +20953,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>C009</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -20968,7 +20968,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-04 16:54</t>
+          <t>2026-09-04 16:17</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -20977,17 +20977,17 @@
         </is>
       </c>
       <c r="G39" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H39" t="n">
-        <v>18000</v>
+        <v>21000</v>
       </c>
       <c r="I39" t="n">
         <v>8</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-09-04 17:13</t>
+          <t>2026-09-04 16:37</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21079,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-09-04 15:50</t>
+          <t>2026-09-04 15:45</t>
         </is>
       </c>
     </row>
@@ -21217,7 +21217,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-09-05 21:05</t>
+          <t>2026-09-05 21:00</t>
         </is>
       </c>
     </row>
@@ -21263,7 +21263,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-09-05 16:25</t>
+          <t>2026-09-05 16:20</t>
         </is>
       </c>
     </row>
@@ -21336,7 +21336,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-07 08:56</t>
+          <t>2026-09-07 09:25</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -21489,7 +21489,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-09-06 18:16</t>
+          <t>2026-09-06 18:11</t>
         </is>
       </c>
     </row>
@@ -21504,7 +21504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21531,7 +21531,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>117 records</t>
+          <t>118 records</t>
         </is>
       </c>
     </row>
@@ -21990,17 +21990,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IT107</t>
+          <t>IT110</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>2000</v>
+        <v>6500</v>
       </c>
       <c r="E26" t="n">
-        <v>6000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="27">
@@ -22011,17 +22011,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>IT114</t>
+          <t>IT107</t>
         </is>
       </c>
       <c r="C27" t="n">
         <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="E27" t="n">
-        <v>10500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="28">
@@ -22032,17 +22032,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IT121</t>
+          <t>IT117</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="E28" t="n">
-        <v>5000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="29">
@@ -22053,38 +22053,38 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IT128</t>
+          <t>IT125</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D29" t="n">
-        <v>2300</v>
+        <v>4000</v>
       </c>
       <c r="E29" t="n">
-        <v>6900</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ORD009</t>
+          <t>ORD010</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>IT120</t>
+          <t>IT136</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="E30" t="n">
-        <v>7000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="31">
@@ -22095,17 +22095,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IT139</t>
+          <t>IT130</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
-        <v>3000</v>
+        <v>8500</v>
       </c>
       <c r="E31" t="n">
-        <v>3000</v>
+        <v>25500</v>
       </c>
     </row>
     <row r="32">
@@ -22116,14 +22116,14 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>IT135</t>
+          <t>IT140</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="E32" t="n">
         <v>6000</v>
@@ -22137,17 +22137,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>IT152</t>
+          <t>IT142</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>6500</v>
+        <v>5000</v>
       </c>
       <c r="E33" t="n">
-        <v>6500</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="34">
@@ -22158,38 +22158,38 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>IT143</t>
+          <t>IT149</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>5000</v>
+        <v>2000</v>
       </c>
       <c r="E34" t="n">
-        <v>10000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ORD012</t>
+          <t>ORD011</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>IT164</t>
+          <t>IT141</t>
         </is>
       </c>
       <c r="C35" t="n">
         <v>1</v>
       </c>
       <c r="D35" t="n">
-        <v>17500</v>
+        <v>6500</v>
       </c>
       <c r="E35" t="n">
-        <v>17500</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="36">
@@ -22200,59 +22200,59 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IT153</t>
+          <t>IT162</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
-        <v>10500</v>
+        <v>7000</v>
       </c>
       <c r="E36" t="n">
-        <v>10500</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ORD013</t>
+          <t>ORD012</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IT013</t>
+          <t>IT161</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E37" t="n">
-        <v>4000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ORD013</t>
+          <t>ORD012</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IT170</t>
+          <t>IT153</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
-        <v>3000</v>
+        <v>10500</v>
       </c>
       <c r="E38" t="n">
-        <v>9000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="39">
@@ -22263,143 +22263,143 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>IT166</t>
+          <t>IT013</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>6500</v>
+        <v>2000</v>
       </c>
       <c r="E39" t="n">
-        <v>19500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ORD014</t>
+          <t>ORD013</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IT028</t>
+          <t>IT170</t>
         </is>
       </c>
       <c r="C40" t="n">
         <v>3</v>
       </c>
       <c r="D40" t="n">
-        <v>2300</v>
+        <v>3000</v>
       </c>
       <c r="E40" t="n">
-        <v>6900</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ORD014</t>
+          <t>ORD013</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IT187</t>
+          <t>IT166</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>2000</v>
+        <v>6500</v>
       </c>
       <c r="E41" t="n">
-        <v>4000</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ORD015</t>
+          <t>ORD014</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IT193</t>
+          <t>IT028</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>3</v>
       </c>
       <c r="D42" t="n">
-        <v>4500</v>
+        <v>2300</v>
       </c>
       <c r="E42" t="n">
-        <v>13500</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ORD015</t>
+          <t>ORD014</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IT196</t>
+          <t>IT187</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D43" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="E43" t="n">
-        <v>9000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ORD016</t>
+          <t>ORD015</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IT201</t>
+          <t>IT193</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>3</v>
       </c>
       <c r="D44" t="n">
-        <v>2500</v>
+        <v>4500</v>
       </c>
       <c r="E44" t="n">
-        <v>7500</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ORD016</t>
+          <t>ORD015</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IT058</t>
+          <t>IT196</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D45" t="n">
-        <v>6500</v>
+        <v>3000</v>
       </c>
       <c r="E45" t="n">
-        <v>13000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="46">
@@ -22410,59 +22410,59 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>IT197</t>
+          <t>IT201</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D46" t="n">
-        <v>5500</v>
+        <v>2500</v>
       </c>
       <c r="E46" t="n">
-        <v>11000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ORD017</t>
+          <t>ORD016</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IT078</t>
+          <t>IT058</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>1300</v>
+        <v>6500</v>
       </c>
       <c r="E47" t="n">
-        <v>3900</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ORD017</t>
+          <t>ORD016</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IT080</t>
+          <t>IT197</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>3000</v>
+        <v>5500</v>
       </c>
       <c r="E48" t="n">
-        <v>9000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="49">
@@ -22473,59 +22473,59 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IT210</t>
+          <t>IT078</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D49" t="n">
-        <v>800</v>
+        <v>1300</v>
       </c>
       <c r="E49" t="n">
-        <v>800</v>
+        <v>3900</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ORD018</t>
+          <t>ORD017</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>IT090</t>
+          <t>IT080</t>
         </is>
       </c>
       <c r="C50" t="n">
         <v>3</v>
       </c>
       <c r="D50" t="n">
-        <v>5000</v>
+        <v>3000</v>
       </c>
       <c r="E50" t="n">
-        <v>15000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ORD018</t>
+          <t>ORD017</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IT088</t>
+          <t>IT210</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D51" t="n">
-        <v>12500</v>
+        <v>800</v>
       </c>
       <c r="E51" t="n">
-        <v>25000</v>
+        <v>800</v>
       </c>
     </row>
     <row r="52">
@@ -22536,112 +22536,112 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>IT215</t>
+          <t>IT090</t>
         </is>
       </c>
       <c r="C52" t="n">
         <v>3</v>
       </c>
       <c r="D52" t="n">
-        <v>6000</v>
+        <v>5000</v>
       </c>
       <c r="E52" t="n">
-        <v>18000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ORD019</t>
+          <t>ORD018</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IT094</t>
+          <t>IT088</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>7500</v>
+        <v>12500</v>
       </c>
       <c r="E53" t="n">
-        <v>15000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ORD019</t>
+          <t>ORD018</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IT221</t>
+          <t>IT215</t>
         </is>
       </c>
       <c r="C54" t="n">
         <v>3</v>
       </c>
       <c r="D54" t="n">
-        <v>5000</v>
+        <v>6000</v>
       </c>
       <c r="E54" t="n">
-        <v>15000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ORD020</t>
+          <t>ORD019</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IT109</t>
+          <t>IT094</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>4000</v>
+        <v>7500</v>
       </c>
       <c r="E55" t="n">
-        <v>4000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ORD020</t>
+          <t>ORD019</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IT236</t>
+          <t>IT221</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="E56" t="n">
-        <v>3000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ORD021</t>
+          <t>ORD020</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IT125</t>
+          <t>IT109</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -22657,64 +22657,64 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ORD021</t>
+          <t>ORD020</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IT118</t>
+          <t>IT236</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D58" t="n">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="E58" t="n">
-        <v>18000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ORD022</t>
+          <t>ORD021</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>IT131</t>
+          <t>IT125</t>
         </is>
       </c>
       <c r="C59" t="n">
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>9000</v>
+        <v>4000</v>
       </c>
       <c r="E59" t="n">
-        <v>9000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ORD022</t>
+          <t>ORD021</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IT138</t>
+          <t>IT118</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D60" t="n">
-        <v>2000</v>
+        <v>6000</v>
       </c>
       <c r="E60" t="n">
-        <v>4000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="61">
@@ -22725,59 +22725,59 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IT136</t>
+          <t>IT131</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D61" t="n">
-        <v>5000</v>
+        <v>9000</v>
       </c>
       <c r="E61" t="n">
-        <v>10000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ORD023</t>
+          <t>ORD022</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IT150</t>
+          <t>IT138</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
         <v>2000</v>
       </c>
       <c r="E62" t="n">
-        <v>2000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ORD023</t>
+          <t>ORD022</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>IT143</t>
+          <t>IT136</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D63" t="n">
         <v>5000</v>
       </c>
       <c r="E63" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="64">
@@ -22788,59 +22788,59 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IT151</t>
+          <t>IT150</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>6500</v>
+        <v>2000</v>
       </c>
       <c r="E64" t="n">
-        <v>19500</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ORD024</t>
+          <t>ORD023</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>IT155</t>
+          <t>IT143</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D65" t="n">
-        <v>8000</v>
+        <v>5000</v>
       </c>
       <c r="E65" t="n">
-        <v>16000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ORD024</t>
+          <t>ORD023</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>IT164</t>
+          <t>IT151</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D66" t="n">
-        <v>17500</v>
+        <v>6500</v>
       </c>
       <c r="E66" t="n">
-        <v>35000</v>
+        <v>19500</v>
       </c>
     </row>
     <row r="67">
@@ -22851,59 +22851,59 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>IT160</t>
+          <t>IT155</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D67" t="n">
-        <v>2000</v>
+        <v>8000</v>
       </c>
       <c r="E67" t="n">
-        <v>6000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ORD025</t>
+          <t>ORD024</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>IT030</t>
+          <t>IT164</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D68" t="n">
-        <v>2500</v>
+        <v>17500</v>
       </c>
       <c r="E68" t="n">
-        <v>7500</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ORD025</t>
+          <t>ORD024</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>IT034</t>
+          <t>IT160</t>
         </is>
       </c>
       <c r="C69" t="n">
         <v>3</v>
       </c>
       <c r="D69" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="E69" t="n">
-        <v>10500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="70">
@@ -22914,59 +22914,59 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>IT170</t>
+          <t>IT030</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D70" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E70" t="n">
-        <v>3000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ORD026</t>
+          <t>ORD025</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>IT02</t>
+          <t>IT034</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D71" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="E71" t="n">
-        <v>10000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ORD026</t>
+          <t>ORD025</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IT024</t>
+          <t>IT170</t>
         </is>
       </c>
       <c r="C72" t="n">
         <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
       <c r="E72" t="n">
-        <v>4500</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="73">
@@ -22977,59 +22977,59 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IT041</t>
+          <t>IT02</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D73" t="n">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="E73" t="n">
-        <v>6000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ORD027</t>
+          <t>ORD026</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>IT049</t>
+          <t>IT024</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D74" t="n">
         <v>4500</v>
       </c>
       <c r="E74" t="n">
-        <v>9000</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ORD027</t>
+          <t>ORD026</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IT050</t>
+          <t>IT041</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D75" t="n">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="E75" t="n">
-        <v>7000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="76">
@@ -23040,59 +23040,59 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IT051</t>
+          <t>IT049</t>
         </is>
       </c>
       <c r="C76" t="n">
         <v>2</v>
       </c>
       <c r="D76" t="n">
-        <v>5500</v>
+        <v>4500</v>
       </c>
       <c r="E76" t="n">
-        <v>11000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ORD028</t>
+          <t>ORD027</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>IT058</t>
+          <t>IT050</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D77" t="n">
-        <v>6500</v>
+        <v>3500</v>
       </c>
       <c r="E77" t="n">
-        <v>6500</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ORD028</t>
+          <t>ORD027</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>IT059</t>
+          <t>IT051</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D78" t="n">
-        <v>6500</v>
+        <v>5500</v>
       </c>
       <c r="E78" t="n">
-        <v>6500</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="79">
@@ -23103,59 +23103,59 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>IT060</t>
+          <t>IT058</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>4000</v>
+        <v>6500</v>
       </c>
       <c r="E79" t="n">
-        <v>8000</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ORD029</t>
+          <t>ORD028</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IT206</t>
+          <t>IT059</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D80" t="n">
-        <v>3500</v>
+        <v>6500</v>
       </c>
       <c r="E80" t="n">
-        <v>10500</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ORD029</t>
+          <t>ORD028</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>IT071</t>
+          <t>IT060</t>
         </is>
       </c>
       <c r="C81" t="n">
         <v>2</v>
       </c>
       <c r="D81" t="n">
-        <v>7500</v>
+        <v>4000</v>
       </c>
       <c r="E81" t="n">
-        <v>15000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="82">
@@ -23166,101 +23166,101 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IT077</t>
+          <t>IT206</t>
         </is>
       </c>
       <c r="C82" t="n">
         <v>3</v>
       </c>
       <c r="D82" t="n">
-        <v>1800</v>
+        <v>3500</v>
       </c>
       <c r="E82" t="n">
-        <v>5400</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ORD030</t>
+          <t>ORD029</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IT216</t>
+          <t>IT071</t>
         </is>
       </c>
       <c r="C83" t="n">
         <v>2</v>
       </c>
       <c r="D83" t="n">
-        <v>6000</v>
+        <v>7500</v>
       </c>
       <c r="E83" t="n">
-        <v>12000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ORD030</t>
+          <t>ORD029</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IT088</t>
+          <t>IT077</t>
         </is>
       </c>
       <c r="C84" t="n">
         <v>3</v>
       </c>
       <c r="D84" t="n">
-        <v>12500</v>
+        <v>1800</v>
       </c>
       <c r="E84" t="n">
-        <v>37500</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ORD031</t>
+          <t>ORD030</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>IT228</t>
+          <t>IT216</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D85" t="n">
-        <v>2500</v>
+        <v>6000</v>
       </c>
       <c r="E85" t="n">
-        <v>7500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ORD031</t>
+          <t>ORD030</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>IT226</t>
+          <t>IT088</t>
         </is>
       </c>
       <c r="C86" t="n">
         <v>3</v>
       </c>
       <c r="D86" t="n">
-        <v>3500</v>
+        <v>12500</v>
       </c>
       <c r="E86" t="n">
-        <v>10500</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="87">
@@ -23271,59 +23271,59 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>IT095</t>
+          <t>IT228</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D87" t="n">
-        <v>5500</v>
+        <v>2500</v>
       </c>
       <c r="E87" t="n">
-        <v>5500</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ORD032</t>
+          <t>ORD031</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>IT108</t>
+          <t>IT226</t>
         </is>
       </c>
       <c r="C88" t="n">
         <v>3</v>
       </c>
       <c r="D88" t="n">
-        <v>1000</v>
+        <v>3500</v>
       </c>
       <c r="E88" t="n">
-        <v>3000</v>
+        <v>10500</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ORD032</t>
+          <t>ORD031</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>IT230</t>
+          <t>IT095</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D89" t="n">
-        <v>2500</v>
+        <v>5500</v>
       </c>
       <c r="E89" t="n">
-        <v>5000</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="90">
@@ -23334,38 +23334,38 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>IT235</t>
+          <t>IT231</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D90" t="n">
-        <v>2000</v>
+        <v>17500</v>
       </c>
       <c r="E90" t="n">
-        <v>2000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ORD033</t>
+          <t>ORD032</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>IT125</t>
+          <t>IT108</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D91" t="n">
-        <v>4000</v>
+        <v>1000</v>
       </c>
       <c r="E91" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="92">
@@ -23376,38 +23376,38 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>IT122</t>
+          <t>IT125</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D92" t="n">
-        <v>3000</v>
+        <v>4000</v>
       </c>
       <c r="E92" t="n">
-        <v>6000</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ORD034</t>
+          <t>ORD033</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>IT139</t>
+          <t>IT120</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D93" t="n">
-        <v>3000</v>
+        <v>3500</v>
       </c>
       <c r="E93" t="n">
-        <v>9000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="94">
@@ -23418,35 +23418,35 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>IT140</t>
+          <t>IT139</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D94" t="n">
         <v>3000</v>
       </c>
       <c r="E94" t="n">
-        <v>9000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ORD035</t>
+          <t>ORD034</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>IT148</t>
+          <t>IT133</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D95" t="n">
-        <v>9000</v>
+        <v>6000</v>
       </c>
       <c r="E95" t="n">
         <v>18000</v>
@@ -23460,17 +23460,17 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>IT146</t>
+          <t>IT148</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D96" t="n">
-        <v>4000</v>
+        <v>9000</v>
       </c>
       <c r="E96" t="n">
-        <v>12000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="97">
@@ -23481,38 +23481,38 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>IT144</t>
+          <t>IT146</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D97" t="n">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="E97" t="n">
-        <v>4500</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ORD036</t>
+          <t>ORD035</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>IT157</t>
+          <t>IT144</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D98" t="n">
-        <v>8500</v>
+        <v>4500</v>
       </c>
       <c r="E98" t="n">
-        <v>25500</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="99">
@@ -23523,38 +23523,38 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>IT155</t>
+          <t>IT157</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D99" t="n">
-        <v>8000</v>
+        <v>8500</v>
       </c>
       <c r="E99" t="n">
-        <v>16000</v>
+        <v>25500</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ORD037</t>
+          <t>ORD036</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>IT009</t>
+          <t>IT155</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D100" t="n">
-        <v>6000</v>
+        <v>8000</v>
       </c>
       <c r="E100" t="n">
-        <v>6000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="101">
@@ -23565,14 +23565,14 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>IT033</t>
+          <t>IT009</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D101" t="n">
-        <v>3000</v>
+        <v>6000</v>
       </c>
       <c r="E101" t="n">
         <v>6000</v>
@@ -23581,22 +23581,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ORD038</t>
+          <t>ORD037</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>IT026</t>
+          <t>IT033</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D102" t="n">
         <v>3000</v>
       </c>
       <c r="E102" t="n">
-        <v>9000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="103">
@@ -23607,38 +23607,38 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>IT178</t>
+          <t>IT026</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D103" t="n">
-        <v>5500</v>
+        <v>3000</v>
       </c>
       <c r="E103" t="n">
-        <v>5500</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ORD039</t>
+          <t>ORD038</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>IT050</t>
+          <t>IT178</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D104" t="n">
-        <v>3500</v>
+        <v>5500</v>
       </c>
       <c r="E104" t="n">
-        <v>7000</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="105">
@@ -23649,17 +23649,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>IT054</t>
+          <t>IT050</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D105" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E105" t="n">
-        <v>7500</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="106">
@@ -23670,38 +23670,38 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>IT194</t>
+          <t>IT054</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D106" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E106" t="n">
-        <v>6000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ORD040</t>
+          <t>ORD039</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>IT067</t>
+          <t>IT194</t>
         </is>
       </c>
       <c r="C107" t="n">
         <v>2</v>
       </c>
       <c r="D107" t="n">
-        <v>3500</v>
+        <v>3000</v>
       </c>
       <c r="E107" t="n">
-        <v>7000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="108">
@@ -23712,38 +23712,38 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>IT065</t>
+          <t>IT067</t>
         </is>
       </c>
       <c r="C108" t="n">
         <v>2</v>
       </c>
       <c r="D108" t="n">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="E108" t="n">
-        <v>5000</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ORD041</t>
+          <t>ORD040</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>IT078</t>
+          <t>IT065</t>
         </is>
       </c>
       <c r="C109" t="n">
         <v>2</v>
       </c>
       <c r="D109" t="n">
-        <v>1300</v>
+        <v>2500</v>
       </c>
       <c r="E109" t="n">
-        <v>2600</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="110">
@@ -23754,38 +23754,38 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>IT080</t>
+          <t>IT078</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D110" t="n">
-        <v>3000</v>
+        <v>1300</v>
       </c>
       <c r="E110" t="n">
-        <v>3000</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ORD042</t>
+          <t>ORD041</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>IT091</t>
+          <t>IT080</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D111" t="n">
-        <v>4000</v>
+        <v>3000</v>
       </c>
       <c r="E111" t="n">
-        <v>8000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="112">
@@ -23796,17 +23796,17 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>IT218</t>
+          <t>IT091</t>
         </is>
       </c>
       <c r="C112" t="n">
         <v>2</v>
       </c>
       <c r="D112" t="n">
-        <v>20000</v>
+        <v>4000</v>
       </c>
       <c r="E112" t="n">
-        <v>40000</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="113">
@@ -23817,38 +23817,38 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>IT090</t>
+          <t>IT218</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D113" t="n">
-        <v>5000</v>
+        <v>20000</v>
       </c>
       <c r="E113" t="n">
-        <v>5000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ORD043</t>
+          <t>ORD042</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>IT096</t>
+          <t>IT090</t>
         </is>
       </c>
       <c r="C114" t="n">
         <v>1</v>
       </c>
       <c r="D114" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="E114" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="115">
@@ -23859,17 +23859,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>IT098</t>
+          <t>IT096</t>
         </is>
       </c>
       <c r="C115" t="n">
         <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>7000</v>
+        <v>10000</v>
       </c>
       <c r="E115" t="n">
-        <v>7000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="116">
@@ -23880,38 +23880,38 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>IT225</t>
+          <t>IT098</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D116" t="n">
-        <v>2500</v>
+        <v>7000</v>
       </c>
       <c r="E116" t="n">
-        <v>7500</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ORD044</t>
+          <t>ORD043</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>IT105</t>
+          <t>IT225</t>
         </is>
       </c>
       <c r="C117" t="n">
         <v>3</v>
       </c>
       <c r="D117" t="n">
-        <v>9500</v>
+        <v>2500</v>
       </c>
       <c r="E117" t="n">
-        <v>28500</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="118">
@@ -23922,17 +23922,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>IT110</t>
+          <t>IT105</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D118" t="n">
-        <v>6500</v>
+        <v>9500</v>
       </c>
       <c r="E118" t="n">
-        <v>13000</v>
+        <v>28500</v>
       </c>
     </row>
     <row r="119">
@@ -23943,38 +23943,38 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>IT106</t>
+          <t>IT110</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D119" t="n">
-        <v>7000</v>
+        <v>6500</v>
       </c>
       <c r="E119" t="n">
-        <v>7000</v>
+        <v>13000</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ORD045</t>
+          <t>ORD044</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>IT117</t>
+          <t>IT106</t>
         </is>
       </c>
       <c r="C120" t="n">
         <v>1</v>
       </c>
       <c r="D120" t="n">
-        <v>3500</v>
+        <v>7000</v>
       </c>
       <c r="E120" t="n">
-        <v>3500</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="121">
@@ -23985,17 +23985,17 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>IT121</t>
+          <t>IT117</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D121" t="n">
-        <v>5000</v>
+        <v>3500</v>
       </c>
       <c r="E121" t="n">
-        <v>15000</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="122">
@@ -24006,16 +24006,37 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
+          <t>IT121</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>3</v>
+      </c>
+      <c r="D122" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E122" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ORD045</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
           <t>IT120</t>
         </is>
       </c>
-      <c r="C122" t="n">
-        <v>1</v>
-      </c>
-      <c r="D122" t="n">
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
+      <c r="D123" t="n">
         <v>3500</v>
       </c>
-      <c r="E122" t="n">
+      <c r="E123" t="n">
         <v>3500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace two emoji that recent Unicode blocks leave unrendered
</commit_message>
<xml_diff>
--- a/Chowly - Seed Data.xlsx
+++ b/Chowly - Seed Data.xlsx
@@ -1340,7 +1340,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-07 09:16</t>
+          <t>2026-09-07 14:13</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1368,7 +1368,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-07 09:18</t>
+          <t>2026-09-07 14:15</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1644,7 +1644,7 @@
       <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-07 09:07</t>
+          <t>2026-09-07 14:04</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-09-07 09:37</t>
+          <t>2026-09-07 14:34</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-07 09:29</t>
+          <t>2026-09-07 14:26</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -13411,7 +13411,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>🫖</t>
+          <t>🍵</t>
         </is>
       </c>
     </row>
@@ -14354,7 +14354,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>🫖</t>
+          <t>🍵</t>
         </is>
       </c>
     </row>
@@ -14805,7 +14805,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>🫖</t>
+          <t>🍵</t>
         </is>
       </c>
     </row>
@@ -17593,7 +17593,7 @@
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>🫐</t>
+          <t>🍓</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18700,7 @@
       </c>
       <c r="I225" t="inlineStr">
         <is>
-          <t>🫖</t>
+          <t>🍵</t>
         </is>
       </c>
     </row>
@@ -19233,7 +19233,7 @@
       </c>
       <c r="I238" t="inlineStr">
         <is>
-          <t>🫖</t>
+          <t>🍵</t>
         </is>
       </c>
     </row>
@@ -19528,7 +19528,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-07 09:07</t>
+          <t>2026-09-07 14:04</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -19892,7 +19892,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-07 09:09</t>
+          <t>2026-09-07 14:06</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -20164,7 +20164,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-07 09:35</t>
+          <t>2026-09-07 14:32</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -20252,7 +20252,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-07 09:14</t>
+          <t>2026-09-07 14:11</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -20294,7 +20294,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-07 09:16</t>
+          <t>2026-09-07 14:13</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -20704,7 +20704,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-07 09:03</t>
+          <t>2026-09-07 14:00</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -20746,7 +20746,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-07 09:34</t>
+          <t>2026-09-07 14:31</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -20880,7 +20880,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-07 09:40</t>
+          <t>2026-09-07 14:37</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -21336,7 +21336,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-07 09:25</t>
+          <t>2026-09-07 14:22</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">

</xml_diff>